<commit_message>
Update dated price quotes and source check report
</commit_message>
<xml_diff>
--- a/assets/pbs-weekly.xlsx
+++ b/assets/pbs-weekly.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\192.168.21.33\d\00 COMMON FOLDER AT LOCAL SERVER\00 SPI New Base 2015-16\SPI New Base-2015-16\SPI 2026\10. October 2026\22.10.2026\SPI Email 22.10.2026\E-Office\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\192.168.21.33\d\00 COMMON FOLDER AT LOCAL SERVER\00 SPI New Base 2015-16\SPI New Base-2015-16\SPI 2026\10. October 2026\29.10.2026\SPI Email 29.10.2026\E-Office\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF934EC7-AE5A-46A2-9E5E-53CE510F57DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6B53524-3A01-4DFC-91B9-B290576A5D6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{68A2838D-D4B6-4512-A2A7-5B35B075D955}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{A5E87162-F82E-4B89-B659-D047582E000F}"/>
   </bookViews>
   <sheets>
     <sheet name="Appendix-A" sheetId="11" r:id="rId1"/>
@@ -61,7 +61,7 @@
     <t>CONSUMER PRICES OF ESSENTIAL ITEMS</t>
   </si>
   <si>
-    <t>PRICES ON 22-10-2026</t>
+    <t>PRICES ON 29-10-2026</t>
   </si>
   <si>
     <t>Islamabad (01)</t>
@@ -421,7 +421,7 @@
     <t>Quetta</t>
   </si>
   <si>
-    <t>A: Retail Prices of Fertilizers (50 kg/bag) for the Week Ended on 22-10-2026</t>
+    <t>A: Retail Prices of Fertilizers (50 kg/bag) for the Week Ended on 29-10-2026</t>
   </si>
   <si>
     <t>No.</t>
@@ -430,10 +430,10 @@
     <t>Description</t>
   </si>
   <si>
-    <t>Average Price for                                                22-10-26 15-10-26 23-10-25</t>
+    <t>Average Price for                                                29-10-26 22-10-26 30-10-25</t>
   </si>
   <si>
-    <t>% Change over                 15-10-26 23-10-25</t>
+    <t>% Change over                 22-10-26 30-10-25</t>
   </si>
   <si>
     <t>Sona Urea</t>
@@ -475,7 +475,7 @@
     <t>Khuz-dar</t>
   </si>
   <si>
-    <t>B: Retail Prices of Cement (50 kg/bag) for the Week Ended on 22-10-2026</t>
+    <t>B: Retail Prices of Cement (50 kg/bag) for the Week Ended on 29-10-2026</t>
   </si>
   <si>
     <t>Avg. Price per litre</t>
@@ -487,23 +487,23 @@
     <t>Avg. Price per kg</t>
   </si>
   <si>
-    <t>C: Prices of CNG (per litre for Punjab and per kg otherwise) for the Week Ended on 22-10-2026</t>
+    <t>C: Prices of CNG (per litre for Punjab and per kg otherwise) for the Week Ended on 29-10-2026</t>
   </si>
   <si>
-    <t>D: Wage Rates for the Week Ended on 22-10-2026</t>
+    <t>D: Wage Rates for the Week Ended on 29-10-2026</t>
   </si>
   <si>
-    <t>E: Wheat Rates for the Week Ended on 22.10.2026</t>
+    <t>E: Wheat Rates for the Week Ended on 29.10.2026</t>
   </si>
   <si>
     <t>Khuzdar</t>
   </si>
   <si>
     <t>Average Price for
-22.10.2026     15.10.2026</t>
+29.10.2026     22.10.2026</t>
   </si>
   <si>
-    <t>% Change over               15.10.2026</t>
+    <t>% Change over               22.10.2026</t>
   </si>
   <si>
     <t>Wheat</t>
@@ -1112,7 +1112,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{037DF315-4EC9-405D-9F19-F9FD1F66B04A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F308F6B9-B4D2-45CE-AEFF-7C6D8E0A69A3}">
   <dimension ref="A1:Y179"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1428,7 +1428,7 @@
         <v>3240</v>
       </c>
       <c r="E7" s="6">
-        <v>3286.54</v>
+        <v>3278.77</v>
       </c>
       <c r="F7" s="6">
         <v>3333.33</v>
@@ -1437,10 +1437,10 @@
         <v>2200</v>
       </c>
       <c r="H7" s="6">
-        <v>2945.37</v>
+        <v>2937.39</v>
       </c>
       <c r="I7" s="6">
-        <v>3333.33</v>
+        <v>3306.66</v>
       </c>
       <c r="J7" s="6">
         <v>2200</v>
@@ -1479,13 +1479,13 @@
         <v>3000</v>
       </c>
       <c r="V7" s="6">
-        <v>2800</v>
+        <v>2200</v>
       </c>
       <c r="W7" s="6">
-        <v>2800</v>
+        <v>2421.3200000000002</v>
       </c>
       <c r="X7" s="6">
-        <v>2800</v>
+        <v>2933</v>
       </c>
       <c r="Y7" s="7">
         <v>1</v>
@@ -1656,22 +1656,22 @@
         <v>23</v>
       </c>
       <c r="D10" s="6">
-        <v>120</v>
+        <v>130</v>
       </c>
       <c r="E10" s="6">
-        <v>120</v>
+        <v>130</v>
       </c>
       <c r="F10" s="6">
-        <v>120</v>
+        <v>130</v>
       </c>
       <c r="G10" s="6">
-        <v>120</v>
+        <v>130</v>
       </c>
       <c r="H10" s="6">
-        <v>120</v>
+        <v>130</v>
       </c>
       <c r="I10" s="6">
-        <v>120</v>
+        <v>130</v>
       </c>
       <c r="J10" s="6">
         <v>120</v>
@@ -1887,67 +1887,67 @@
         <v>20</v>
       </c>
       <c r="D13" s="6">
-        <v>420</v>
+        <v>410</v>
       </c>
       <c r="E13" s="6">
-        <v>437.94</v>
+        <v>429.54</v>
       </c>
       <c r="F13" s="6">
-        <v>470</v>
+        <v>460</v>
       </c>
       <c r="G13" s="6">
         <v>420</v>
       </c>
       <c r="H13" s="6">
-        <v>435.24</v>
+        <v>429.6</v>
       </c>
       <c r="I13" s="6">
-        <v>450</v>
+        <v>440</v>
       </c>
       <c r="J13" s="6">
+        <v>403</v>
+      </c>
+      <c r="K13" s="6">
+        <v>403</v>
+      </c>
+      <c r="L13" s="6">
+        <v>403</v>
+      </c>
+      <c r="M13" s="6">
+        <v>398</v>
+      </c>
+      <c r="N13" s="6">
+        <v>398</v>
+      </c>
+      <c r="O13" s="6">
+        <v>398</v>
+      </c>
+      <c r="P13" s="6">
+        <v>388</v>
+      </c>
+      <c r="Q13" s="6">
+        <v>388</v>
+      </c>
+      <c r="R13" s="6">
+        <v>388</v>
+      </c>
+      <c r="S13" s="6">
         <v>405</v>
       </c>
-      <c r="K13" s="6">
+      <c r="T13" s="6">
         <v>405</v>
       </c>
-      <c r="L13" s="6">
+      <c r="U13" s="6">
         <v>405</v>
       </c>
-      <c r="M13" s="6">
-        <v>396</v>
-      </c>
-      <c r="N13" s="6">
-        <v>396</v>
-      </c>
-      <c r="O13" s="6">
-        <v>396</v>
-      </c>
-      <c r="P13" s="6">
-        <v>398</v>
-      </c>
-      <c r="Q13" s="6">
-        <v>398</v>
-      </c>
-      <c r="R13" s="6">
-        <v>398</v>
-      </c>
-      <c r="S13" s="6">
-        <v>440</v>
-      </c>
-      <c r="T13" s="6">
-        <v>440</v>
-      </c>
-      <c r="U13" s="6">
-        <v>440</v>
-      </c>
       <c r="V13" s="6">
+        <v>410</v>
+      </c>
+      <c r="W13" s="6">
+        <v>411.66</v>
+      </c>
+      <c r="X13" s="6">
         <v>415</v>
-      </c>
-      <c r="W13" s="6">
-        <v>416.66</v>
-      </c>
-      <c r="X13" s="6">
-        <v>420</v>
       </c>
       <c r="Y13" s="7">
         <v>7</v>
@@ -1991,10 +1991,10 @@
         <v>220</v>
       </c>
       <c r="M14" s="6">
-        <v>180</v>
+        <v>230</v>
       </c>
       <c r="N14" s="6">
-        <v>211.95</v>
+        <v>230</v>
       </c>
       <c r="O14" s="6">
         <v>230</v>
@@ -2068,10 +2068,10 @@
         <v>240</v>
       </c>
       <c r="M15" s="6">
-        <v>190</v>
+        <v>240</v>
       </c>
       <c r="N15" s="6">
-        <v>222.02</v>
+        <v>240</v>
       </c>
       <c r="O15" s="6">
         <v>240</v>
@@ -2136,13 +2136,13 @@
         <v>1100</v>
       </c>
       <c r="J16" s="6">
-        <v>1160</v>
+        <v>1100</v>
       </c>
       <c r="K16" s="6">
-        <v>1163.32</v>
+        <v>1100</v>
       </c>
       <c r="L16" s="6">
-        <v>1170</v>
+        <v>1100</v>
       </c>
       <c r="M16" s="6">
         <v>1180</v>
@@ -2195,28 +2195,28 @@
         <v>32</v>
       </c>
       <c r="D17" s="6">
-        <v>268</v>
+        <v>240</v>
       </c>
       <c r="E17" s="6">
-        <v>269.67</v>
+        <v>252.4</v>
       </c>
       <c r="F17" s="6">
-        <v>270</v>
+        <v>260</v>
       </c>
       <c r="G17" s="6">
-        <v>268</v>
+        <v>240</v>
       </c>
       <c r="H17" s="6">
-        <v>269.06</v>
+        <v>252.26</v>
       </c>
       <c r="I17" s="6">
-        <v>270</v>
+        <v>260</v>
       </c>
       <c r="J17" s="6">
-        <v>250</v>
+        <v>240</v>
       </c>
       <c r="K17" s="6">
-        <v>250</v>
+        <v>246.62</v>
       </c>
       <c r="L17" s="6">
         <v>250</v>
@@ -2231,31 +2231,31 @@
         <v>265</v>
       </c>
       <c r="P17" s="6">
-        <v>267</v>
+        <v>239</v>
       </c>
       <c r="Q17" s="6">
-        <v>267</v>
+        <v>239</v>
       </c>
       <c r="R17" s="6">
-        <v>267</v>
+        <v>239</v>
       </c>
       <c r="S17" s="6">
-        <v>267</v>
+        <v>260</v>
       </c>
       <c r="T17" s="6">
-        <v>267</v>
+        <v>260</v>
       </c>
       <c r="U17" s="6">
-        <v>267</v>
+        <v>260</v>
       </c>
       <c r="V17" s="6">
-        <v>267</v>
+        <v>239</v>
       </c>
       <c r="W17" s="6">
-        <v>267</v>
+        <v>239</v>
       </c>
       <c r="X17" s="6">
-        <v>267</v>
+        <v>239</v>
       </c>
       <c r="Y17" s="7">
         <v>11</v>
@@ -2444,13 +2444,13 @@
         <v>1605</v>
       </c>
       <c r="J20" s="6">
-        <v>1580</v>
+        <v>1605</v>
       </c>
       <c r="K20" s="6">
-        <v>1580</v>
+        <v>1605</v>
       </c>
       <c r="L20" s="6">
-        <v>1580</v>
+        <v>1605</v>
       </c>
       <c r="M20" s="6">
         <v>1580</v>
@@ -2548,13 +2548,13 @@
         <v>625</v>
       </c>
       <c r="S21" s="6">
-        <v>615</v>
+        <v>625</v>
       </c>
       <c r="T21" s="6">
-        <v>615</v>
+        <v>625</v>
       </c>
       <c r="U21" s="6">
-        <v>615</v>
+        <v>625</v>
       </c>
       <c r="V21" s="6">
         <v>625</v>
@@ -2583,16 +2583,16 @@
         <v>180</v>
       </c>
       <c r="E22" s="6">
-        <v>216.09</v>
+        <v>215.38</v>
       </c>
       <c r="F22" s="6">
         <v>260</v>
       </c>
       <c r="G22" s="6">
-        <v>200</v>
+        <v>180</v>
       </c>
       <c r="H22" s="6">
-        <v>207.83</v>
+        <v>197.79</v>
       </c>
       <c r="I22" s="6">
         <v>220</v>
@@ -2619,10 +2619,10 @@
         <v>140</v>
       </c>
       <c r="Q22" s="6">
-        <v>151.11000000000001</v>
+        <v>156.78</v>
       </c>
       <c r="R22" s="6">
-        <v>170</v>
+        <v>180</v>
       </c>
       <c r="S22" s="6">
         <v>130</v>
@@ -2675,13 +2675,13 @@
         <v>310</v>
       </c>
       <c r="J23" s="6">
-        <v>240</v>
+        <v>230</v>
       </c>
       <c r="K23" s="6">
-        <v>240</v>
+        <v>230</v>
       </c>
       <c r="L23" s="6">
-        <v>240</v>
+        <v>230</v>
       </c>
       <c r="M23" s="6">
         <v>260</v>
@@ -2942,10 +2942,10 @@
         <v>250</v>
       </c>
       <c r="V26" s="6">
-        <v>270</v>
+        <v>280</v>
       </c>
       <c r="W26" s="6">
-        <v>276.63</v>
+        <v>280</v>
       </c>
       <c r="X26" s="6">
         <v>280</v>
@@ -2968,19 +2968,19 @@
         <v>60</v>
       </c>
       <c r="E27" s="6">
-        <v>72.62</v>
+        <v>79.849999999999994</v>
       </c>
       <c r="F27" s="6">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="G27" s="6">
         <v>55</v>
       </c>
       <c r="H27" s="6">
-        <v>67.17</v>
+        <v>75.599999999999994</v>
       </c>
       <c r="I27" s="6">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="J27" s="6">
         <v>50</v>
@@ -3001,10 +3001,10 @@
         <v>70</v>
       </c>
       <c r="P27" s="6">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="Q27" s="6">
-        <v>56.69</v>
+        <v>63.42</v>
       </c>
       <c r="R27" s="6">
         <v>70</v>
@@ -3045,19 +3045,19 @@
         <v>200</v>
       </c>
       <c r="E28" s="6">
-        <v>234.17</v>
+        <v>227.06</v>
       </c>
       <c r="F28" s="6">
-        <v>270</v>
+        <v>250</v>
       </c>
       <c r="G28" s="6">
-        <v>220</v>
+        <v>200</v>
       </c>
       <c r="H28" s="6">
-        <v>233.49</v>
+        <v>225.04</v>
       </c>
       <c r="I28" s="6">
-        <v>250</v>
+        <v>240</v>
       </c>
       <c r="J28" s="6">
         <v>200</v>
@@ -3069,28 +3069,28 @@
         <v>200</v>
       </c>
       <c r="M28" s="6">
+        <v>220</v>
+      </c>
+      <c r="N28" s="6">
+        <v>220</v>
+      </c>
+      <c r="O28" s="6">
+        <v>220</v>
+      </c>
+      <c r="P28" s="6">
         <v>200</v>
       </c>
-      <c r="N28" s="6">
-        <v>200</v>
-      </c>
-      <c r="O28" s="6">
-        <v>200</v>
-      </c>
-      <c r="P28" s="6">
-        <v>190</v>
-      </c>
       <c r="Q28" s="6">
-        <v>199.35</v>
+        <v>209.36</v>
       </c>
       <c r="R28" s="6">
-        <v>220</v>
+        <v>230</v>
       </c>
       <c r="S28" s="6">
         <v>180</v>
       </c>
       <c r="T28" s="6">
-        <v>186.43</v>
+        <v>193.1</v>
       </c>
       <c r="U28" s="6">
         <v>200</v>
@@ -3099,10 +3099,10 @@
         <v>190</v>
       </c>
       <c r="W28" s="6">
-        <v>190</v>
+        <v>193.28</v>
       </c>
       <c r="X28" s="6">
-        <v>190</v>
+        <v>200</v>
       </c>
       <c r="Y28" s="7">
         <v>22</v>
@@ -3119,67 +3119,67 @@
         <v>20</v>
       </c>
       <c r="D29" s="6">
-        <v>140</v>
+        <v>150</v>
       </c>
       <c r="E29" s="6">
-        <v>167.43</v>
+        <v>172.76</v>
       </c>
       <c r="F29" s="6">
         <v>200</v>
       </c>
       <c r="G29" s="6">
+        <v>160</v>
+      </c>
+      <c r="H29" s="6">
+        <v>170.15</v>
+      </c>
+      <c r="I29" s="6">
+        <v>180</v>
+      </c>
+      <c r="J29" s="6">
+        <v>180</v>
+      </c>
+      <c r="K29" s="6">
+        <v>180</v>
+      </c>
+      <c r="L29" s="6">
+        <v>180</v>
+      </c>
+      <c r="M29" s="6">
+        <v>160</v>
+      </c>
+      <c r="N29" s="6">
+        <v>160</v>
+      </c>
+      <c r="O29" s="6">
+        <v>160</v>
+      </c>
+      <c r="P29" s="6">
         <v>140</v>
       </c>
-      <c r="H29" s="6">
-        <v>154.41</v>
-      </c>
-      <c r="I29" s="6">
+      <c r="Q29" s="6">
+        <v>150.96</v>
+      </c>
+      <c r="R29" s="6">
         <v>170</v>
       </c>
-      <c r="J29" s="6">
-        <v>120</v>
-      </c>
-      <c r="K29" s="6">
-        <v>120</v>
-      </c>
-      <c r="L29" s="6">
-        <v>120</v>
-      </c>
-      <c r="M29" s="6">
-        <v>100</v>
-      </c>
-      <c r="N29" s="6">
-        <v>100</v>
-      </c>
-      <c r="O29" s="6">
-        <v>100</v>
-      </c>
-      <c r="P29" s="6">
-        <v>100</v>
-      </c>
-      <c r="Q29" s="6">
-        <v>106.72</v>
-      </c>
-      <c r="R29" s="6">
-        <v>120</v>
-      </c>
       <c r="S29" s="6">
-        <v>100</v>
+        <v>130</v>
       </c>
       <c r="T29" s="6">
-        <v>112.92</v>
+        <v>130</v>
       </c>
       <c r="U29" s="6">
-        <v>120</v>
+        <v>130</v>
       </c>
       <c r="V29" s="6">
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="W29" s="6">
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="X29" s="6">
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="Y29" s="7">
         <v>23</v>
@@ -3196,22 +3196,22 @@
         <v>20</v>
       </c>
       <c r="D30" s="6">
+        <v>140</v>
+      </c>
+      <c r="E30" s="6">
+        <v>142.06</v>
+      </c>
+      <c r="F30" s="6">
         <v>145</v>
       </c>
-      <c r="E30" s="6">
-        <v>148.31</v>
-      </c>
-      <c r="F30" s="6">
-        <v>150</v>
-      </c>
       <c r="G30" s="6">
+        <v>140</v>
+      </c>
+      <c r="H30" s="6">
+        <v>142.31</v>
+      </c>
+      <c r="I30" s="6">
         <v>145</v>
-      </c>
-      <c r="H30" s="6">
-        <v>148.99</v>
-      </c>
-      <c r="I30" s="6">
-        <v>150</v>
       </c>
       <c r="J30" s="6">
         <v>140</v>
@@ -3330,10 +3330,10 @@
         <v>220</v>
       </c>
       <c r="W31" s="6">
-        <v>221.65</v>
+        <v>220</v>
       </c>
       <c r="X31" s="6">
-        <v>225</v>
+        <v>220</v>
       </c>
       <c r="Y31" s="7">
         <v>25</v>
@@ -3552,7 +3552,7 @@
         <v>300</v>
       </c>
       <c r="T34" s="6">
-        <v>315.82</v>
+        <v>332.47</v>
       </c>
       <c r="U34" s="6">
         <v>350</v>
@@ -3851,7 +3851,7 @@
         <v>70</v>
       </c>
       <c r="Q38" s="6">
-        <v>71.349999999999994</v>
+        <v>71.8</v>
       </c>
       <c r="R38" s="6">
         <v>80</v>
@@ -4505,67 +4505,67 @@
         <v>66</v>
       </c>
       <c r="D47" s="6">
-        <v>7.66</v>
+        <v>7.36</v>
       </c>
       <c r="E47" s="6">
-        <v>7.66</v>
+        <v>7.36</v>
       </c>
       <c r="F47" s="6">
-        <v>7.66</v>
+        <v>7.36</v>
       </c>
       <c r="G47" s="6">
-        <v>7.66</v>
+        <v>7.36</v>
       </c>
       <c r="H47" s="6">
-        <v>7.66</v>
+        <v>7.36</v>
       </c>
       <c r="I47" s="6">
-        <v>7.66</v>
+        <v>7.36</v>
       </c>
       <c r="J47" s="6">
-        <v>7.66</v>
+        <v>7.36</v>
       </c>
       <c r="K47" s="6">
-        <v>7.66</v>
+        <v>7.36</v>
       </c>
       <c r="L47" s="6">
-        <v>7.66</v>
+        <v>7.36</v>
       </c>
       <c r="M47" s="6">
-        <v>7.66</v>
+        <v>7.36</v>
       </c>
       <c r="N47" s="6">
-        <v>7.66</v>
+        <v>7.36</v>
       </c>
       <c r="O47" s="6">
-        <v>7.66</v>
+        <v>7.36</v>
       </c>
       <c r="P47" s="6">
-        <v>7.66</v>
+        <v>7.36</v>
       </c>
       <c r="Q47" s="6">
-        <v>7.66</v>
+        <v>7.36</v>
       </c>
       <c r="R47" s="6">
-        <v>7.66</v>
+        <v>7.36</v>
       </c>
       <c r="S47" s="6">
-        <v>7.66</v>
+        <v>7.36</v>
       </c>
       <c r="T47" s="6">
-        <v>7.66</v>
+        <v>7.36</v>
       </c>
       <c r="U47" s="6">
-        <v>7.66</v>
+        <v>7.36</v>
       </c>
       <c r="V47" s="6">
-        <v>7.66</v>
+        <v>7.36</v>
       </c>
       <c r="W47" s="6">
-        <v>7.66</v>
+        <v>7.36</v>
       </c>
       <c r="X47" s="6">
-        <v>7.66</v>
+        <v>7.36</v>
       </c>
       <c r="Y47" s="7">
         <v>41</v>
@@ -4713,13 +4713,13 @@
         <v>1800</v>
       </c>
       <c r="V49" s="6">
-        <v>1450</v>
+        <v>1500</v>
       </c>
       <c r="W49" s="6">
-        <v>1483.14</v>
+        <v>1516.48</v>
       </c>
       <c r="X49" s="6">
-        <v>1500</v>
+        <v>1550</v>
       </c>
       <c r="Y49" s="7">
         <v>43</v>
@@ -4967,67 +4967,67 @@
         <v>75</v>
       </c>
       <c r="D53" s="6">
-        <v>380.88</v>
+        <v>379.48</v>
       </c>
       <c r="E53" s="6">
-        <v>380.88</v>
+        <v>379.48</v>
       </c>
       <c r="F53" s="6">
-        <v>380.88</v>
+        <v>379.48</v>
       </c>
       <c r="G53" s="6">
-        <v>380.24</v>
+        <v>379.34</v>
       </c>
       <c r="H53" s="6">
-        <v>380.73</v>
+        <v>379.36</v>
       </c>
       <c r="I53" s="6">
-        <v>380.86</v>
+        <v>379.46</v>
       </c>
       <c r="J53" s="6">
-        <v>381.54</v>
+        <v>380.25</v>
       </c>
       <c r="K53" s="6">
-        <v>381.54</v>
+        <v>380.25</v>
       </c>
       <c r="L53" s="6">
-        <v>381.54</v>
+        <v>380.25</v>
       </c>
       <c r="M53" s="6">
-        <v>381.9</v>
+        <v>381.05</v>
       </c>
       <c r="N53" s="6">
-        <v>381.9</v>
+        <v>381.05</v>
       </c>
       <c r="O53" s="6">
-        <v>381.9</v>
+        <v>381.05</v>
       </c>
       <c r="P53" s="6">
-        <v>379.31</v>
+        <v>377.91</v>
       </c>
       <c r="Q53" s="6">
-        <v>379.31</v>
+        <v>377.91</v>
       </c>
       <c r="R53" s="6">
-        <v>379.31</v>
+        <v>377.91</v>
       </c>
       <c r="S53" s="6">
-        <v>380.74</v>
+        <v>379.34</v>
       </c>
       <c r="T53" s="6">
-        <v>380.74</v>
+        <v>379.34</v>
       </c>
       <c r="U53" s="6">
-        <v>380.74</v>
+        <v>379.34</v>
       </c>
       <c r="V53" s="6">
-        <v>382.81</v>
+        <v>381.41</v>
       </c>
       <c r="W53" s="6">
-        <v>382.81</v>
+        <v>381.41</v>
       </c>
       <c r="X53" s="6">
-        <v>382.81</v>
+        <v>381.41</v>
       </c>
       <c r="Y53" s="7">
         <v>47</v>
@@ -5044,67 +5044,67 @@
         <v>75</v>
       </c>
       <c r="D54" s="6">
-        <v>391.66</v>
+        <v>401.37</v>
       </c>
       <c r="E54" s="6">
-        <v>391.66</v>
+        <v>401.37</v>
       </c>
       <c r="F54" s="6">
-        <v>391.66</v>
+        <v>401.37</v>
       </c>
       <c r="G54" s="6">
-        <v>390.75</v>
+        <v>400.08</v>
       </c>
       <c r="H54" s="6">
-        <v>391.52</v>
+        <v>401.21</v>
       </c>
       <c r="I54" s="6">
-        <v>391.76</v>
+        <v>401.47</v>
       </c>
       <c r="J54" s="6">
-        <v>392.34</v>
+        <v>402.16</v>
       </c>
       <c r="K54" s="6">
-        <v>392.34</v>
+        <v>402.16</v>
       </c>
       <c r="L54" s="6">
-        <v>392.34</v>
+        <v>402.16</v>
       </c>
       <c r="M54" s="6">
-        <v>392.7</v>
+        <v>403.1</v>
       </c>
       <c r="N54" s="6">
-        <v>392.7</v>
+        <v>403.1</v>
       </c>
       <c r="O54" s="6">
-        <v>392.7</v>
+        <v>403.1</v>
       </c>
       <c r="P54" s="6">
-        <v>390.11</v>
+        <v>399.82</v>
       </c>
       <c r="Q54" s="6">
-        <v>390.11</v>
+        <v>399.82</v>
       </c>
       <c r="R54" s="6">
-        <v>390.11</v>
+        <v>399.82</v>
       </c>
       <c r="S54" s="6">
-        <v>391.54</v>
+        <v>401.25</v>
       </c>
       <c r="T54" s="6">
-        <v>391.74</v>
+        <v>401.25</v>
       </c>
       <c r="U54" s="6">
-        <v>391.94</v>
+        <v>401.25</v>
       </c>
       <c r="V54" s="6">
-        <v>393.61</v>
+        <v>403.32</v>
       </c>
       <c r="W54" s="6">
-        <v>393.61</v>
+        <v>403.32</v>
       </c>
       <c r="X54" s="6">
-        <v>393.61</v>
+        <v>403.32</v>
       </c>
       <c r="Y54" s="7">
         <v>48</v>
@@ -5142,46 +5142,46 @@
         <v>6418.5</v>
       </c>
       <c r="K55" s="6">
-        <v>6457.17</v>
+        <v>6418.5</v>
       </c>
       <c r="L55" s="6">
-        <v>6535.2</v>
+        <v>6418.5</v>
       </c>
       <c r="M55" s="6">
-        <v>7002</v>
+        <v>6419</v>
       </c>
       <c r="N55" s="6">
-        <v>7002</v>
+        <v>6419</v>
       </c>
       <c r="O55" s="6">
-        <v>7002</v>
+        <v>6419</v>
       </c>
       <c r="P55" s="6">
-        <v>6418.5</v>
+        <v>6068.4</v>
       </c>
       <c r="Q55" s="6">
-        <v>6457.17</v>
+        <v>6107.05</v>
       </c>
       <c r="R55" s="6">
-        <v>6535.2</v>
+        <v>6185.1</v>
       </c>
       <c r="S55" s="6">
-        <v>6000</v>
+        <v>6400</v>
       </c>
       <c r="T55" s="6">
-        <v>6263.79</v>
+        <v>6400</v>
       </c>
       <c r="U55" s="6">
         <v>6400</v>
       </c>
       <c r="V55" s="6">
-        <v>5700</v>
+        <v>5900</v>
       </c>
       <c r="W55" s="6">
-        <v>5700</v>
+        <v>5900</v>
       </c>
       <c r="X55" s="6">
-        <v>5700</v>
+        <v>5900</v>
       </c>
       <c r="Y55" s="7">
         <v>49</v>
@@ -5683,10 +5683,10 @@
         <v>2946.66</v>
       </c>
       <c r="J65" s="6">
-        <v>3300</v>
+        <v>3200</v>
       </c>
       <c r="K65" s="6">
-        <v>3412.18</v>
+        <v>3371.02</v>
       </c>
       <c r="L65" s="6">
         <v>3540</v>
@@ -5701,19 +5701,19 @@
         <v>3400</v>
       </c>
       <c r="P65" s="6">
-        <v>3120</v>
+        <v>3160</v>
       </c>
       <c r="Q65" s="6">
-        <v>3120</v>
+        <v>3160</v>
       </c>
       <c r="R65" s="6">
-        <v>3120</v>
+        <v>3160</v>
       </c>
       <c r="S65" s="6">
-        <v>3300</v>
+        <v>3250</v>
       </c>
       <c r="T65" s="6">
-        <v>3300</v>
+        <v>3266.58</v>
       </c>
       <c r="U65" s="6">
         <v>3300</v>
@@ -5722,7 +5722,7 @@
         <v>2520</v>
       </c>
       <c r="W65" s="6">
-        <v>3038.96</v>
+        <v>3060.48</v>
       </c>
       <c r="X65" s="6">
         <v>3300</v>
@@ -6127,67 +6127,67 @@
         <v>20</v>
       </c>
       <c r="D71" s="6">
-        <v>440</v>
+        <v>435</v>
       </c>
       <c r="E71" s="6">
-        <v>440</v>
+        <v>435</v>
       </c>
       <c r="F71" s="6">
-        <v>440</v>
+        <v>435</v>
       </c>
       <c r="G71" s="6">
-        <v>410</v>
+        <v>400</v>
       </c>
       <c r="H71" s="6">
-        <v>410</v>
+        <v>406.64</v>
       </c>
       <c r="I71" s="6">
         <v>410</v>
       </c>
       <c r="J71" s="6">
-        <v>500</v>
+        <v>440</v>
       </c>
       <c r="K71" s="6">
-        <v>510.23</v>
+        <v>452.29</v>
       </c>
       <c r="L71" s="6">
-        <v>520</v>
+        <v>480</v>
       </c>
       <c r="M71" s="6">
-        <v>480</v>
+        <v>440</v>
       </c>
       <c r="N71" s="6">
-        <v>486.23</v>
+        <v>442.48</v>
       </c>
       <c r="O71" s="6">
-        <v>490</v>
+        <v>450</v>
       </c>
       <c r="P71" s="6">
-        <v>460</v>
+        <v>410</v>
       </c>
       <c r="Q71" s="6">
-        <v>460</v>
+        <v>429.53</v>
       </c>
       <c r="R71" s="6">
-        <v>460</v>
+        <v>450</v>
       </c>
       <c r="S71" s="6">
-        <v>460</v>
+        <v>440</v>
       </c>
       <c r="T71" s="6">
-        <v>460</v>
+        <v>443.31</v>
       </c>
       <c r="U71" s="6">
-        <v>460</v>
+        <v>450</v>
       </c>
       <c r="V71" s="6">
-        <v>440</v>
+        <v>430</v>
       </c>
       <c r="W71" s="6">
-        <v>440</v>
+        <v>430</v>
       </c>
       <c r="X71" s="6">
-        <v>440</v>
+        <v>430</v>
       </c>
       <c r="Y71" s="7">
         <v>7</v>
@@ -6444,19 +6444,19 @@
         <v>260</v>
       </c>
       <c r="G75" s="6">
-        <v>250</v>
+        <v>240</v>
       </c>
       <c r="H75" s="6">
-        <v>250</v>
+        <v>246.62</v>
       </c>
       <c r="I75" s="6">
         <v>250</v>
       </c>
       <c r="J75" s="6">
-        <v>270</v>
+        <v>250</v>
       </c>
       <c r="K75" s="6">
-        <v>273.45</v>
+        <v>265</v>
       </c>
       <c r="L75" s="6">
         <v>280</v>
@@ -6465,7 +6465,7 @@
         <v>240</v>
       </c>
       <c r="N75" s="6">
-        <v>249.02</v>
+        <v>248.17</v>
       </c>
       <c r="O75" s="6">
         <v>260</v>
@@ -6480,19 +6480,19 @@
         <v>260</v>
       </c>
       <c r="S75" s="6">
-        <v>250</v>
+        <v>240</v>
       </c>
       <c r="T75" s="6">
-        <v>256.62</v>
+        <v>253.15</v>
       </c>
       <c r="U75" s="6">
         <v>260</v>
       </c>
       <c r="V75" s="6">
-        <v>260</v>
+        <v>250</v>
       </c>
       <c r="W75" s="6">
-        <v>276.58</v>
+        <v>272.06</v>
       </c>
       <c r="X75" s="6">
         <v>280</v>
@@ -6764,7 +6764,7 @@
         <v>615</v>
       </c>
       <c r="K79" s="6">
-        <v>616.80999999999995</v>
+        <v>618.32000000000005</v>
       </c>
       <c r="L79" s="6">
         <v>625</v>
@@ -6841,7 +6841,7 @@
         <v>80</v>
       </c>
       <c r="K80" s="6">
-        <v>112.21</v>
+        <v>111.59</v>
       </c>
       <c r="L80" s="6">
         <v>150</v>
@@ -6918,7 +6918,7 @@
         <v>260</v>
       </c>
       <c r="K81" s="6">
-        <v>278.24</v>
+        <v>278.77999999999997</v>
       </c>
       <c r="L81" s="6">
         <v>320</v>
@@ -6995,7 +6995,7 @@
         <v>320</v>
       </c>
       <c r="K82" s="6">
-        <v>355.33</v>
+        <v>356.43</v>
       </c>
       <c r="L82" s="6">
         <v>400</v>
@@ -7128,28 +7128,28 @@
         <v>20</v>
       </c>
       <c r="D84" s="6">
+        <v>310</v>
+      </c>
+      <c r="E84" s="6">
+        <v>321.02999999999997</v>
+      </c>
+      <c r="F84" s="6">
+        <v>330</v>
+      </c>
+      <c r="G84" s="6">
+        <v>260</v>
+      </c>
+      <c r="H84" s="6">
+        <v>266.5</v>
+      </c>
+      <c r="I84" s="6">
+        <v>280</v>
+      </c>
+      <c r="J84" s="6">
         <v>300</v>
       </c>
-      <c r="E84" s="6">
-        <v>306.56</v>
-      </c>
-      <c r="F84" s="6">
-        <v>320</v>
-      </c>
-      <c r="G84" s="6">
-        <v>240</v>
-      </c>
-      <c r="H84" s="6">
-        <v>249.87</v>
-      </c>
-      <c r="I84" s="6">
-        <v>260</v>
-      </c>
-      <c r="J84" s="6">
-        <v>290</v>
-      </c>
       <c r="K84" s="6">
-        <v>312.79000000000002</v>
+        <v>316.12</v>
       </c>
       <c r="L84" s="6">
         <v>340</v>
@@ -7164,13 +7164,13 @@
         <v>320</v>
       </c>
       <c r="P84" s="6">
-        <v>280</v>
+        <v>300</v>
       </c>
       <c r="Q84" s="6">
-        <v>280</v>
+        <v>300</v>
       </c>
       <c r="R84" s="6">
-        <v>280</v>
+        <v>300</v>
       </c>
       <c r="S84" s="6">
         <v>290</v>
@@ -7217,16 +7217,16 @@
         <v>30</v>
       </c>
       <c r="H85" s="6">
-        <v>33.020000000000003</v>
+        <v>39.15</v>
       </c>
       <c r="I85" s="6">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="J85" s="6">
         <v>40</v>
       </c>
       <c r="K85" s="6">
-        <v>55.9</v>
+        <v>58.3</v>
       </c>
       <c r="L85" s="6">
         <v>70</v>
@@ -7253,7 +7253,7 @@
         <v>30</v>
       </c>
       <c r="T85" s="6">
-        <v>31.58</v>
+        <v>33.25</v>
       </c>
       <c r="U85" s="6">
         <v>35</v>
@@ -7262,7 +7262,7 @@
         <v>50</v>
       </c>
       <c r="W85" s="6">
-        <v>57.62</v>
+        <v>55.33</v>
       </c>
       <c r="X85" s="6">
         <v>60</v>
@@ -7300,10 +7300,10 @@
         <v>200</v>
       </c>
       <c r="J86" s="6">
-        <v>150</v>
+        <v>160</v>
       </c>
       <c r="K86" s="6">
-        <v>175.79</v>
+        <v>179.92</v>
       </c>
       <c r="L86" s="6">
         <v>200</v>
@@ -7327,22 +7327,22 @@
         <v>160</v>
       </c>
       <c r="S86" s="6">
-        <v>160</v>
+        <v>170</v>
       </c>
       <c r="T86" s="6">
-        <v>163.27000000000001</v>
+        <v>176.6</v>
       </c>
       <c r="U86" s="6">
-        <v>170</v>
+        <v>180</v>
       </c>
       <c r="V86" s="6">
-        <v>220</v>
+        <v>210</v>
       </c>
       <c r="W86" s="6">
-        <v>225.45</v>
+        <v>218.82</v>
       </c>
       <c r="X86" s="6">
-        <v>240</v>
+        <v>230</v>
       </c>
       <c r="Y86" s="7">
         <v>22</v>
@@ -7359,49 +7359,49 @@
         <v>20</v>
       </c>
       <c r="D87" s="6">
-        <v>70</v>
+        <v>100</v>
       </c>
       <c r="E87" s="6">
-        <v>83.92</v>
+        <v>108.44</v>
       </c>
       <c r="F87" s="6">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="G87" s="6">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="H87" s="6">
-        <v>78.3</v>
+        <v>126.33</v>
       </c>
       <c r="I87" s="6">
-        <v>100</v>
+        <v>140</v>
       </c>
       <c r="J87" s="6">
-        <v>50</v>
+        <v>80</v>
       </c>
       <c r="K87" s="6">
-        <v>75.02</v>
+        <v>117.32</v>
       </c>
       <c r="L87" s="6">
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="M87" s="6">
-        <v>50</v>
+        <v>120</v>
       </c>
       <c r="N87" s="6">
-        <v>53.13</v>
+        <v>133.94</v>
       </c>
       <c r="O87" s="6">
-        <v>60</v>
+        <v>140</v>
       </c>
       <c r="P87" s="6">
-        <v>50</v>
+        <v>120</v>
       </c>
       <c r="Q87" s="6">
-        <v>50</v>
+        <v>120</v>
       </c>
       <c r="R87" s="6">
-        <v>50</v>
+        <v>120</v>
       </c>
       <c r="S87" s="6">
         <v>70</v>
@@ -7413,10 +7413,10 @@
         <v>80</v>
       </c>
       <c r="V87" s="6">
-        <v>120</v>
+        <v>130</v>
       </c>
       <c r="W87" s="6">
-        <v>126.41</v>
+        <v>134.35</v>
       </c>
       <c r="X87" s="6">
         <v>140</v>
@@ -7457,7 +7457,7 @@
         <v>135</v>
       </c>
       <c r="K88" s="6">
-        <v>142.21</v>
+        <v>141.46</v>
       </c>
       <c r="L88" s="6">
         <v>150</v>
@@ -7765,7 +7765,7 @@
         <v>320</v>
       </c>
       <c r="K92" s="6">
-        <v>411.08</v>
+        <v>413.15</v>
       </c>
       <c r="L92" s="6">
         <v>560</v>
@@ -8745,67 +8745,67 @@
         <v>66</v>
       </c>
       <c r="D105" s="6">
-        <v>7.66</v>
+        <v>7.36</v>
       </c>
       <c r="E105" s="6">
-        <v>7.66</v>
+        <v>7.36</v>
       </c>
       <c r="F105" s="6">
-        <v>7.66</v>
+        <v>7.36</v>
       </c>
       <c r="G105" s="6">
-        <v>7.66</v>
+        <v>7.36</v>
       </c>
       <c r="H105" s="6">
-        <v>7.66</v>
+        <v>7.36</v>
       </c>
       <c r="I105" s="6">
-        <v>7.66</v>
+        <v>7.36</v>
       </c>
       <c r="J105" s="6">
-        <v>7.66</v>
+        <v>7.36</v>
       </c>
       <c r="K105" s="6">
-        <v>7.66</v>
+        <v>7.36</v>
       </c>
       <c r="L105" s="6">
-        <v>7.66</v>
+        <v>7.36</v>
       </c>
       <c r="M105" s="6">
-        <v>7.66</v>
+        <v>7.36</v>
       </c>
       <c r="N105" s="6">
-        <v>7.66</v>
+        <v>7.36</v>
       </c>
       <c r="O105" s="6">
-        <v>7.66</v>
+        <v>7.36</v>
       </c>
       <c r="P105" s="6">
-        <v>7.66</v>
+        <v>7.36</v>
       </c>
       <c r="Q105" s="6">
-        <v>7.66</v>
+        <v>7.36</v>
       </c>
       <c r="R105" s="6">
-        <v>7.66</v>
+        <v>7.36</v>
       </c>
       <c r="S105" s="6">
-        <v>7.66</v>
+        <v>7.36</v>
       </c>
       <c r="T105" s="6">
-        <v>7.66</v>
+        <v>7.36</v>
       </c>
       <c r="U105" s="6">
-        <v>7.66</v>
+        <v>7.36</v>
       </c>
       <c r="V105" s="6">
-        <v>7.66</v>
+        <v>7.36</v>
       </c>
       <c r="W105" s="6">
-        <v>7.66</v>
+        <v>7.36</v>
       </c>
       <c r="X105" s="6">
-        <v>7.66</v>
+        <v>7.36</v>
       </c>
       <c r="Y105" s="7">
         <v>41</v>
@@ -8929,10 +8929,10 @@
         <v>1450</v>
       </c>
       <c r="N107" s="6">
-        <v>1483.14</v>
+        <v>1499.86</v>
       </c>
       <c r="O107" s="6">
-        <v>1500</v>
+        <v>1550</v>
       </c>
       <c r="P107" s="6">
         <v>1100</v>
@@ -9207,67 +9207,67 @@
         <v>75</v>
       </c>
       <c r="D111" s="6">
-        <v>380.14</v>
+        <v>379.3</v>
       </c>
       <c r="E111" s="6">
-        <v>380.67</v>
+        <v>379.69</v>
       </c>
       <c r="F111" s="6">
-        <v>381.66</v>
+        <v>380.56</v>
       </c>
       <c r="G111" s="6">
-        <v>382.61</v>
+        <v>381.21</v>
       </c>
       <c r="H111" s="6">
-        <v>382.89</v>
+        <v>381.61</v>
       </c>
       <c r="I111" s="6">
-        <v>383.1</v>
+        <v>381.92</v>
       </c>
       <c r="J111" s="6">
-        <v>380.74</v>
+        <v>379.34</v>
       </c>
       <c r="K111" s="6">
-        <v>380.74</v>
+        <v>379.34</v>
       </c>
       <c r="L111" s="6">
-        <v>380.74</v>
+        <v>379.34</v>
       </c>
       <c r="M111" s="6">
-        <v>383.13</v>
+        <v>381.41</v>
       </c>
       <c r="N111" s="6">
-        <v>383.52</v>
+        <v>381.86</v>
       </c>
       <c r="O111" s="6">
-        <v>383.96</v>
+        <v>382.56</v>
       </c>
       <c r="P111" s="6">
-        <v>380.93</v>
+        <v>379.53</v>
       </c>
       <c r="Q111" s="6">
-        <v>380.93</v>
+        <v>379.53</v>
       </c>
       <c r="R111" s="6">
-        <v>380.93</v>
+        <v>379.53</v>
       </c>
       <c r="S111" s="6">
-        <v>382.14</v>
+        <v>381.47</v>
       </c>
       <c r="T111" s="6">
-        <v>382.14</v>
+        <v>381.47</v>
       </c>
       <c r="U111" s="6">
-        <v>382.14</v>
+        <v>381.47</v>
       </c>
       <c r="V111" s="6">
-        <v>384</v>
+        <v>379.3</v>
       </c>
       <c r="W111" s="6">
-        <v>384</v>
+        <v>379.3</v>
       </c>
       <c r="X111" s="6">
-        <v>384</v>
+        <v>379.3</v>
       </c>
       <c r="Y111" s="7">
         <v>47</v>
@@ -9284,67 +9284,67 @@
         <v>75</v>
       </c>
       <c r="D112" s="6">
-        <v>391.36</v>
+        <v>401.2</v>
       </c>
       <c r="E112" s="6">
-        <v>391.83</v>
+        <v>401.59</v>
       </c>
       <c r="F112" s="6">
-        <v>392.59</v>
+        <v>402.45</v>
       </c>
       <c r="G112" s="6">
-        <v>393.41</v>
+        <v>403.12</v>
       </c>
       <c r="H112" s="6">
-        <v>393.82</v>
+        <v>403.53</v>
       </c>
       <c r="I112" s="6">
-        <v>394.1</v>
+        <v>403.86</v>
       </c>
       <c r="J112" s="6">
-        <v>391.54</v>
+        <v>401.25</v>
       </c>
       <c r="K112" s="6">
-        <v>391.54</v>
+        <v>401.25</v>
       </c>
       <c r="L112" s="6">
-        <v>391.54</v>
+        <v>401.25</v>
       </c>
       <c r="M112" s="6">
-        <v>393.61</v>
+        <v>403.32</v>
       </c>
       <c r="N112" s="6">
-        <v>394.08</v>
+        <v>403.75</v>
       </c>
       <c r="O112" s="6">
-        <v>394.7</v>
+        <v>404.4</v>
       </c>
       <c r="P112" s="6">
-        <v>391.73</v>
+        <v>401.44</v>
       </c>
       <c r="Q112" s="6">
-        <v>391.73</v>
+        <v>401.44</v>
       </c>
       <c r="R112" s="6">
-        <v>391.73</v>
+        <v>401.44</v>
       </c>
       <c r="S112" s="6">
-        <v>392.14</v>
+        <v>402.62</v>
       </c>
       <c r="T112" s="6">
-        <v>392.41</v>
+        <v>402.62</v>
       </c>
       <c r="U112" s="6">
-        <v>392.94</v>
+        <v>402.62</v>
       </c>
       <c r="V112" s="6">
-        <v>391.2</v>
+        <v>401.3</v>
       </c>
       <c r="W112" s="6">
-        <v>391.2</v>
+        <v>401.3</v>
       </c>
       <c r="X112" s="6">
-        <v>391.2</v>
+        <v>401.3</v>
       </c>
       <c r="Y112" s="7">
         <v>48</v>
@@ -9361,13 +9361,13 @@
         <v>23</v>
       </c>
       <c r="D113" s="6">
-        <v>6300</v>
+        <v>6180</v>
       </c>
       <c r="E113" s="6">
-        <v>6402.12</v>
+        <v>6181.67</v>
       </c>
       <c r="F113" s="6">
-        <v>6415</v>
+        <v>6185</v>
       </c>
       <c r="G113" s="6">
         <v>7000</v>
@@ -9379,46 +9379,46 @@
         <v>7100</v>
       </c>
       <c r="J113" s="6">
-        <v>6301</v>
+        <v>5835</v>
       </c>
       <c r="K113" s="6">
-        <v>6410.81</v>
+        <v>5998.99</v>
       </c>
       <c r="L113" s="6">
-        <v>6535</v>
+        <v>6185</v>
       </c>
       <c r="M113" s="6">
+        <v>6068.4</v>
+      </c>
+      <c r="N113" s="6">
+        <v>6107.05</v>
+      </c>
+      <c r="O113" s="6">
         <v>6185.1</v>
       </c>
-      <c r="N113" s="6">
-        <v>6262.48</v>
-      </c>
-      <c r="O113" s="6">
-        <v>6418.5</v>
-      </c>
       <c r="P113" s="6">
-        <v>6190</v>
+        <v>5840</v>
       </c>
       <c r="Q113" s="6">
-        <v>6190</v>
+        <v>5840</v>
       </c>
       <c r="R113" s="6">
-        <v>6190</v>
+        <v>5840</v>
       </c>
       <c r="S113" s="6">
-        <v>5600</v>
+        <v>6150</v>
       </c>
       <c r="T113" s="6">
-        <v>5600</v>
+        <v>6150</v>
       </c>
       <c r="U113" s="6">
-        <v>5600</v>
+        <v>6150</v>
       </c>
       <c r="V113" s="6">
-        <v>6301.8</v>
+        <v>6068.4</v>
       </c>
       <c r="W113" s="6">
-        <v>6558.33</v>
+        <v>6340.59</v>
       </c>
       <c r="X113" s="6">
         <v>6768.6</v>
@@ -9901,22 +9901,22 @@
         <v>18</v>
       </c>
       <c r="D123" s="6">
-        <v>3150</v>
+        <v>3100</v>
       </c>
       <c r="E123" s="6">
-        <v>3150</v>
+        <v>3166.31</v>
       </c>
       <c r="F123" s="6">
-        <v>3150</v>
+        <v>3200</v>
       </c>
       <c r="G123" s="6">
-        <v>3150</v>
+        <v>3170</v>
       </c>
       <c r="H123" s="6">
-        <v>3164.99</v>
+        <v>3184.99</v>
       </c>
       <c r="I123" s="6">
-        <v>3180</v>
+        <v>3200</v>
       </c>
       <c r="J123" s="6">
         <v>3200</v>
@@ -9931,24 +9931,24 @@
         <v>2200</v>
       </c>
       <c r="N123" s="6">
-        <v>2976.12</v>
+        <v>2951.46</v>
       </c>
       <c r="O123" s="6">
         <v>3540</v>
       </c>
       <c r="P123" s="6">
-        <v>2946.72</v>
+        <v>2976.12</v>
       </c>
       <c r="Q123" s="6">
-        <v>2180.5</v>
+        <v>2188.42</v>
       </c>
       <c r="R123" s="6">
         <f t="shared" ref="R123:R154" si="0">ROUND(N123/P123* 100 - 100,2)</f>
-        <v>1</v>
+        <v>-0.83</v>
       </c>
       <c r="S123" s="6">
         <f t="shared" ref="S123:S154" si="1">ROUND(N123/Q123* 100 - 100,2)</f>
-        <v>36.49</v>
+        <v>34.869999999999997</v>
       </c>
       <c r="T123" s="6">
         <v>2109.1799999999998</v>
@@ -9989,13 +9989,13 @@
         <v>140</v>
       </c>
       <c r="G124" s="6">
-        <v>270</v>
+        <v>280</v>
       </c>
       <c r="H124" s="6">
-        <v>279.93</v>
+        <v>289.93</v>
       </c>
       <c r="I124" s="6">
-        <v>290</v>
+        <v>300</v>
       </c>
       <c r="J124" s="6">
         <v>240</v>
@@ -10010,24 +10010,24 @@
         <v>140</v>
       </c>
       <c r="N124" s="6">
-        <v>214.76</v>
+        <v>215.2</v>
       </c>
       <c r="O124" s="6">
         <v>300</v>
       </c>
       <c r="P124" s="6">
-        <v>215.52</v>
+        <v>214.76</v>
       </c>
       <c r="Q124" s="6">
         <v>216.89</v>
       </c>
       <c r="R124" s="6">
         <f t="shared" si="0"/>
-        <v>-0.35</v>
+        <v>0.2</v>
       </c>
       <c r="S124" s="6">
         <f t="shared" si="1"/>
-        <v>-0.98</v>
+        <v>-0.78</v>
       </c>
       <c r="T124" s="6">
         <v>214.54</v>
@@ -10068,13 +10068,13 @@
         <v>170</v>
       </c>
       <c r="G125" s="6">
-        <v>160</v>
+        <v>150</v>
       </c>
       <c r="H125" s="6">
-        <v>169.88</v>
+        <v>159.87</v>
       </c>
       <c r="I125" s="6">
-        <v>180</v>
+        <v>170</v>
       </c>
       <c r="J125" s="6">
         <v>150</v>
@@ -10089,24 +10089,24 @@
         <v>110</v>
       </c>
       <c r="N125" s="6">
-        <v>155.07</v>
+        <v>154.4</v>
       </c>
       <c r="O125" s="6">
         <v>200</v>
       </c>
       <c r="P125" s="6">
-        <v>154.88999999999999</v>
+        <v>155.07</v>
       </c>
       <c r="Q125" s="6">
-        <v>157.4</v>
+        <v>157.21</v>
       </c>
       <c r="R125" s="6">
         <f t="shared" si="0"/>
-        <v>0.12</v>
+        <v>-0.43</v>
       </c>
       <c r="S125" s="6">
         <f t="shared" si="1"/>
-        <v>-1.48</v>
+        <v>-1.79</v>
       </c>
       <c r="T125" s="6">
         <v>155.74</v>
@@ -10159,33 +10159,33 @@
         <v>110</v>
       </c>
       <c r="K126" s="6">
-        <v>110</v>
+        <v>116.57</v>
       </c>
       <c r="L126" s="6">
-        <v>110</v>
+        <v>120</v>
       </c>
       <c r="M126" s="6">
         <v>100</v>
       </c>
       <c r="N126" s="6">
-        <v>122.04</v>
+        <v>123.62</v>
       </c>
       <c r="O126" s="6">
         <v>140</v>
       </c>
       <c r="P126" s="6">
-        <v>120.05</v>
+        <v>122.04</v>
       </c>
       <c r="Q126" s="6">
         <v>110.12</v>
       </c>
       <c r="R126" s="6">
         <f t="shared" si="0"/>
-        <v>1.66</v>
+        <v>1.29</v>
       </c>
       <c r="S126" s="6">
         <f t="shared" si="1"/>
-        <v>10.82</v>
+        <v>12.26</v>
       </c>
       <c r="T126" s="6">
         <v>112.09</v>
@@ -10253,14 +10253,14 @@
         <v>1600</v>
       </c>
       <c r="P127" s="6">
-        <v>1275.6300000000001</v>
+        <v>1279.6199999999999</v>
       </c>
       <c r="Q127" s="6">
         <v>1141.48</v>
       </c>
       <c r="R127" s="6">
         <f t="shared" si="0"/>
-        <v>0.31</v>
+        <v>0</v>
       </c>
       <c r="S127" s="6">
         <f t="shared" si="1"/>
@@ -10332,14 +10332,14 @@
         <v>3000</v>
       </c>
       <c r="P128" s="6">
-        <v>2400.2600000000002</v>
+        <v>2401.65</v>
       </c>
       <c r="Q128" s="6">
         <v>2094.59</v>
       </c>
       <c r="R128" s="6">
         <f t="shared" si="0"/>
-        <v>0.06</v>
+        <v>0</v>
       </c>
       <c r="S128" s="6">
         <f t="shared" si="1"/>
@@ -10375,54 +10375,54 @@
         <v>20</v>
       </c>
       <c r="D129" s="6">
-        <v>455</v>
+        <v>435</v>
       </c>
       <c r="E129" s="6">
-        <v>455</v>
+        <v>435</v>
       </c>
       <c r="F129" s="6">
-        <v>455</v>
+        <v>435</v>
       </c>
       <c r="G129" s="6">
-        <v>430</v>
+        <v>460</v>
       </c>
       <c r="H129" s="6">
-        <v>439.96</v>
+        <v>471.62</v>
       </c>
       <c r="I129" s="6">
-        <v>450</v>
+        <v>480</v>
       </c>
       <c r="J129" s="6">
-        <v>550</v>
+        <v>540</v>
       </c>
       <c r="K129" s="6">
-        <v>550</v>
+        <v>540</v>
       </c>
       <c r="L129" s="6">
-        <v>550</v>
+        <v>540</v>
       </c>
       <c r="M129" s="6">
-        <v>396</v>
+        <v>388</v>
       </c>
       <c r="N129" s="6">
+        <v>431.15</v>
+      </c>
+      <c r="O129" s="6">
+        <v>540</v>
+      </c>
+      <c r="P129" s="6">
         <v>444.27</v>
       </c>
-      <c r="O129" s="6">
-        <v>550</v>
-      </c>
-      <c r="P129" s="6">
-        <v>395.98</v>
-      </c>
       <c r="Q129" s="6">
-        <v>319.64</v>
+        <v>327.32</v>
       </c>
       <c r="R129" s="6">
         <f t="shared" si="0"/>
-        <v>12.2</v>
+        <v>-2.95</v>
       </c>
       <c r="S129" s="6">
         <f t="shared" si="1"/>
-        <v>38.99</v>
+        <v>31.72</v>
       </c>
       <c r="T129" s="6">
         <v>385.92</v>
@@ -10484,7 +10484,7 @@
         <v>170</v>
       </c>
       <c r="N130" s="6">
-        <v>218.92</v>
+        <v>219.98</v>
       </c>
       <c r="O130" s="6">
         <v>280</v>
@@ -10497,11 +10497,11 @@
       </c>
       <c r="R130" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.48</v>
       </c>
       <c r="S130" s="6">
         <f t="shared" si="1"/>
-        <v>7.88</v>
+        <v>8.4</v>
       </c>
       <c r="T130" s="6">
         <v>204.78</v>
@@ -10560,10 +10560,10 @@
         <v>240</v>
       </c>
       <c r="M131" s="6">
-        <v>190</v>
+        <v>200</v>
       </c>
       <c r="N131" s="6">
-        <v>257.05</v>
+        <v>258.23</v>
       </c>
       <c r="O131" s="6">
         <v>400</v>
@@ -10572,15 +10572,15 @@
         <v>257.05</v>
       </c>
       <c r="Q131" s="6">
-        <v>238.49</v>
+        <v>238.55</v>
       </c>
       <c r="R131" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.46</v>
       </c>
       <c r="S131" s="6">
         <f t="shared" si="1"/>
-        <v>7.78</v>
+        <v>8.25</v>
       </c>
       <c r="T131" s="6">
         <v>240.43</v>
@@ -10642,24 +10642,24 @@
         <v>1100</v>
       </c>
       <c r="N132" s="6">
-        <v>1147.9100000000001</v>
+        <v>1144.1400000000001</v>
       </c>
       <c r="O132" s="6">
         <v>1200</v>
       </c>
       <c r="P132" s="6">
-        <v>1152.27</v>
+        <v>1147.9100000000001</v>
       </c>
       <c r="Q132" s="6">
-        <v>1112.43</v>
+        <v>1114.83</v>
       </c>
       <c r="R132" s="6">
         <f t="shared" si="0"/>
-        <v>-0.38</v>
+        <v>-0.33</v>
       </c>
       <c r="S132" s="6">
         <f t="shared" si="1"/>
-        <v>3.19</v>
+        <v>2.63</v>
       </c>
       <c r="T132" s="6">
         <v>1123.76</v>
@@ -10694,10 +10694,10 @@
         <v>250</v>
       </c>
       <c r="E133" s="6">
-        <v>253.29</v>
+        <v>250</v>
       </c>
       <c r="F133" s="6">
-        <v>260</v>
+        <v>250</v>
       </c>
       <c r="G133" s="6">
         <v>240</v>
@@ -10718,27 +10718,27 @@
         <v>280</v>
       </c>
       <c r="M133" s="6">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="N133" s="6">
-        <v>261.86</v>
+        <v>254.51</v>
       </c>
       <c r="O133" s="6">
         <v>280</v>
       </c>
       <c r="P133" s="6">
-        <v>263.39</v>
+        <v>261.86</v>
       </c>
       <c r="Q133" s="6">
-        <v>336.34</v>
+        <v>347.24</v>
       </c>
       <c r="R133" s="6">
         <f t="shared" si="0"/>
-        <v>-0.57999999999999996</v>
+        <v>-2.81</v>
       </c>
       <c r="S133" s="6">
         <f t="shared" si="1"/>
-        <v>-22.14</v>
+        <v>-26.7</v>
       </c>
       <c r="T133" s="6">
         <v>285.7</v>
@@ -10806,18 +10806,18 @@
         <v>720</v>
       </c>
       <c r="P134" s="6">
-        <v>568</v>
+        <v>569.55999999999995</v>
       </c>
       <c r="Q134" s="6">
-        <v>539.66999999999996</v>
+        <v>540.14</v>
       </c>
       <c r="R134" s="6">
         <f t="shared" si="0"/>
-        <v>0.27</v>
+        <v>0</v>
       </c>
       <c r="S134" s="6">
         <f t="shared" si="1"/>
-        <v>5.54</v>
+        <v>5.45</v>
       </c>
       <c r="T134" s="6">
         <v>543.98</v>
@@ -10885,18 +10885,18 @@
         <v>3115</v>
       </c>
       <c r="P135" s="6">
-        <v>3092.88</v>
+        <v>3095.81</v>
       </c>
       <c r="Q135" s="6">
-        <v>2895.93</v>
+        <v>2914.51</v>
       </c>
       <c r="R135" s="6">
         <f t="shared" si="0"/>
-        <v>0.09</v>
+        <v>0</v>
       </c>
       <c r="S135" s="6">
         <f t="shared" si="1"/>
-        <v>6.9</v>
+        <v>6.22</v>
       </c>
       <c r="T135" s="6">
         <v>2960.42</v>
@@ -10928,13 +10928,13 @@
         <v>23</v>
       </c>
       <c r="D136" s="6">
-        <v>1500</v>
+        <v>1550</v>
       </c>
       <c r="E136" s="6">
-        <v>1500</v>
+        <v>1550</v>
       </c>
       <c r="F136" s="6">
-        <v>1500</v>
+        <v>1550</v>
       </c>
       <c r="G136" s="6">
         <v>1580</v>
@@ -10955,27 +10955,27 @@
         <v>1580</v>
       </c>
       <c r="M136" s="6">
-        <v>1500</v>
+        <v>1515</v>
       </c>
       <c r="N136" s="6">
-        <v>1574.2</v>
+        <v>1578.69</v>
       </c>
       <c r="O136" s="6">
         <v>1605</v>
       </c>
       <c r="P136" s="6">
-        <v>1571.29</v>
+        <v>1574.2</v>
       </c>
       <c r="Q136" s="6">
-        <v>1483.59</v>
+        <v>1489.49</v>
       </c>
       <c r="R136" s="6">
         <f t="shared" si="0"/>
-        <v>0.19</v>
+        <v>0.28999999999999998</v>
       </c>
       <c r="S136" s="6">
         <f t="shared" si="1"/>
-        <v>6.11</v>
+        <v>5.99</v>
       </c>
       <c r="T136" s="6">
         <v>1502.18</v>
@@ -11037,24 +11037,24 @@
         <v>600</v>
       </c>
       <c r="N137" s="6">
-        <v>617.51</v>
+        <v>618.19000000000005</v>
       </c>
       <c r="O137" s="6">
         <v>625</v>
       </c>
       <c r="P137" s="6">
-        <v>613.88</v>
+        <v>617.51</v>
       </c>
       <c r="Q137" s="6">
-        <v>580.66999999999996</v>
+        <v>581.92999999999995</v>
       </c>
       <c r="R137" s="6">
         <f t="shared" si="0"/>
-        <v>0.59</v>
+        <v>0.11</v>
       </c>
       <c r="S137" s="6">
         <f t="shared" si="1"/>
-        <v>6.34</v>
+        <v>6.23</v>
       </c>
       <c r="T137" s="6">
         <v>584.15</v>
@@ -11086,22 +11086,22 @@
         <v>32</v>
       </c>
       <c r="D138" s="6">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="E138" s="6">
-        <v>112.92</v>
+        <v>120</v>
       </c>
       <c r="F138" s="6">
         <v>120</v>
       </c>
       <c r="G138" s="6">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="H138" s="6">
-        <v>99.16</v>
+        <v>84.46</v>
       </c>
       <c r="I138" s="6">
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="J138" s="6">
         <v>150</v>
@@ -11113,27 +11113,27 @@
         <v>150</v>
       </c>
       <c r="M138" s="6">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="N138" s="6">
-        <v>128.09</v>
+        <v>127.18</v>
       </c>
       <c r="O138" s="6">
         <v>260</v>
       </c>
       <c r="P138" s="6">
-        <v>131.26</v>
+        <v>128.09</v>
       </c>
       <c r="Q138" s="6">
-        <v>123.12</v>
+        <v>123.34</v>
       </c>
       <c r="R138" s="6">
         <f t="shared" si="0"/>
-        <v>-2.42</v>
+        <v>-0.71</v>
       </c>
       <c r="S138" s="6">
         <f t="shared" si="1"/>
-        <v>4.04</v>
+        <v>3.11</v>
       </c>
       <c r="T138" s="6">
         <v>161.47999999999999</v>
@@ -11174,13 +11174,13 @@
         <v>240</v>
       </c>
       <c r="G139" s="6">
-        <v>300</v>
+        <v>290</v>
       </c>
       <c r="H139" s="6">
-        <v>309.93</v>
+        <v>299.93</v>
       </c>
       <c r="I139" s="6">
-        <v>320</v>
+        <v>310</v>
       </c>
       <c r="J139" s="6">
         <v>300</v>
@@ -11195,24 +11195,24 @@
         <v>230</v>
       </c>
       <c r="N139" s="6">
-        <v>268.45999999999998</v>
+        <v>267.31</v>
       </c>
       <c r="O139" s="6">
         <v>330</v>
       </c>
       <c r="P139" s="6">
-        <v>268.52999999999997</v>
+        <v>268.45999999999998</v>
       </c>
       <c r="Q139" s="6">
-        <v>295.27999999999997</v>
+        <v>291.73</v>
       </c>
       <c r="R139" s="6">
         <f t="shared" si="0"/>
-        <v>-0.03</v>
+        <v>-0.43</v>
       </c>
       <c r="S139" s="6">
         <f t="shared" si="1"/>
-        <v>-9.08</v>
+        <v>-8.3699999999999992</v>
       </c>
       <c r="T139" s="6">
         <v>277.24</v>
@@ -11274,24 +11274,24 @@
         <v>280</v>
       </c>
       <c r="N140" s="6">
-        <v>355.04</v>
+        <v>355.1</v>
       </c>
       <c r="O140" s="6">
         <v>440</v>
       </c>
       <c r="P140" s="6">
-        <v>354.32</v>
+        <v>355.04</v>
       </c>
       <c r="Q140" s="6">
-        <v>381.95</v>
+        <v>379.47</v>
       </c>
       <c r="R140" s="6">
         <f t="shared" si="0"/>
-        <v>0.2</v>
+        <v>0.02</v>
       </c>
       <c r="S140" s="6">
         <f t="shared" si="1"/>
-        <v>-7.05</v>
+        <v>-6.42</v>
       </c>
       <c r="T140" s="6">
         <v>386.71</v>
@@ -11359,18 +11359,18 @@
         <v>540</v>
       </c>
       <c r="P141" s="6">
-        <v>469.06</v>
+        <v>470.48</v>
       </c>
       <c r="Q141" s="6">
-        <v>448.32</v>
+        <v>447.7</v>
       </c>
       <c r="R141" s="6">
         <f t="shared" si="0"/>
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="S141" s="6">
         <f t="shared" si="1"/>
-        <v>4.9400000000000004</v>
+        <v>5.09</v>
       </c>
       <c r="T141" s="6">
         <v>452.55</v>
@@ -11411,45 +11411,45 @@
         <v>340</v>
       </c>
       <c r="G142" s="6">
-        <v>320</v>
+        <v>330</v>
       </c>
       <c r="H142" s="6">
-        <v>329.94</v>
+        <v>339.94</v>
       </c>
       <c r="I142" s="6">
-        <v>340</v>
+        <v>350</v>
       </c>
       <c r="J142" s="6">
-        <v>300</v>
+        <v>350</v>
       </c>
       <c r="K142" s="6">
-        <v>309.68</v>
+        <v>350</v>
       </c>
       <c r="L142" s="6">
-        <v>330</v>
+        <v>350</v>
       </c>
       <c r="M142" s="6">
-        <v>240</v>
+        <v>250</v>
       </c>
       <c r="N142" s="6">
-        <v>297.5</v>
+        <v>303.77</v>
       </c>
       <c r="O142" s="6">
         <v>370</v>
       </c>
       <c r="P142" s="6">
-        <v>300.29000000000002</v>
+        <v>297.5</v>
       </c>
       <c r="Q142" s="6">
-        <v>298.25</v>
+        <v>293.31</v>
       </c>
       <c r="R142" s="6">
         <f t="shared" si="0"/>
-        <v>-0.93</v>
+        <v>2.11</v>
       </c>
       <c r="S142" s="6">
         <f t="shared" si="1"/>
-        <v>-0.25</v>
+        <v>3.57</v>
       </c>
       <c r="T142" s="6">
         <v>271.91000000000003</v>
@@ -11511,24 +11511,24 @@
         <v>30</v>
       </c>
       <c r="N143" s="6">
+        <v>51.09</v>
+      </c>
+      <c r="O143" s="6">
+        <v>100</v>
+      </c>
+      <c r="P143" s="6">
         <v>49.47</v>
       </c>
-      <c r="O143" s="6">
-        <v>90</v>
-      </c>
-      <c r="P143" s="6">
-        <v>50.16</v>
-      </c>
       <c r="Q143" s="6">
-        <v>83.5</v>
+        <v>83.31</v>
       </c>
       <c r="R143" s="6">
         <f t="shared" si="0"/>
-        <v>-1.38</v>
+        <v>3.27</v>
       </c>
       <c r="S143" s="6">
         <f t="shared" si="1"/>
-        <v>-40.75</v>
+        <v>-38.67</v>
       </c>
       <c r="T143" s="6">
         <v>54.58</v>
@@ -11581,33 +11581,33 @@
         <v>150</v>
       </c>
       <c r="K144" s="6">
-        <v>165.1</v>
+        <v>150</v>
       </c>
       <c r="L144" s="6">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="M144" s="6">
         <v>130</v>
       </c>
       <c r="N144" s="6">
+        <v>189.74</v>
+      </c>
+      <c r="O144" s="6">
+        <v>250</v>
+      </c>
+      <c r="P144" s="6">
         <v>188.57</v>
       </c>
-      <c r="O144" s="6">
-        <v>270</v>
-      </c>
-      <c r="P144" s="6">
-        <v>180.99</v>
-      </c>
       <c r="Q144" s="6">
-        <v>109.12</v>
+        <v>174.09</v>
       </c>
       <c r="R144" s="6">
         <f t="shared" si="0"/>
-        <v>4.1900000000000004</v>
+        <v>0.62</v>
       </c>
       <c r="S144" s="6">
         <f t="shared" si="1"/>
-        <v>72.81</v>
+        <v>8.99</v>
       </c>
       <c r="T144" s="6">
         <v>81.61</v>
@@ -11639,28 +11639,28 @@
         <v>20</v>
       </c>
       <c r="D145" s="6">
+        <v>120</v>
+      </c>
+      <c r="E145" s="6">
+        <v>120</v>
+      </c>
+      <c r="F145" s="6">
+        <v>120</v>
+      </c>
+      <c r="G145" s="6">
+        <v>50</v>
+      </c>
+      <c r="H145" s="6">
+        <v>64.28</v>
+      </c>
+      <c r="I145" s="6">
         <v>80</v>
       </c>
-      <c r="E145" s="6">
-        <v>89.63</v>
-      </c>
-      <c r="F145" s="6">
+      <c r="J145" s="6">
         <v>100</v>
       </c>
-      <c r="G145" s="6">
-        <v>80</v>
-      </c>
-      <c r="H145" s="6">
-        <v>94.51</v>
-      </c>
-      <c r="I145" s="6">
-        <v>110</v>
-      </c>
-      <c r="J145" s="6">
-        <v>60</v>
-      </c>
       <c r="K145" s="6">
-        <v>78.3</v>
+        <v>100</v>
       </c>
       <c r="L145" s="6">
         <v>100</v>
@@ -11669,24 +11669,24 @@
         <v>50</v>
       </c>
       <c r="N145" s="6">
-        <v>93.17</v>
+        <v>125.7</v>
       </c>
       <c r="O145" s="6">
         <v>200</v>
       </c>
       <c r="P145" s="6">
-        <v>119.43</v>
+        <v>93.17</v>
       </c>
       <c r="Q145" s="6">
-        <v>329.45</v>
+        <v>174.55</v>
       </c>
       <c r="R145" s="6">
         <f t="shared" si="0"/>
-        <v>-21.99</v>
+        <v>34.909999999999997</v>
       </c>
       <c r="S145" s="6">
         <f t="shared" si="1"/>
-        <v>-71.72</v>
+        <v>-27.99</v>
       </c>
       <c r="T145" s="6">
         <v>102.1</v>
@@ -11736,28 +11736,28 @@
         <v>142</v>
       </c>
       <c r="J146" s="6">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="K146" s="6">
-        <v>141.65</v>
+        <v>146.65</v>
       </c>
       <c r="L146" s="6">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="M146" s="6">
         <v>130</v>
       </c>
       <c r="N146" s="6">
-        <v>141.61000000000001</v>
+        <v>141.12</v>
       </c>
       <c r="O146" s="6">
         <v>150</v>
       </c>
       <c r="P146" s="6">
-        <v>142.11000000000001</v>
+        <v>141.61000000000001</v>
       </c>
       <c r="Q146" s="6">
-        <v>188.81</v>
+        <v>188.69</v>
       </c>
       <c r="R146" s="6">
         <f t="shared" si="0"/>
@@ -11765,7 +11765,7 @@
       </c>
       <c r="S146" s="6">
         <f t="shared" si="1"/>
-        <v>-25</v>
+        <v>-25.21</v>
       </c>
       <c r="T146" s="6">
         <v>165.93</v>
@@ -11827,24 +11827,24 @@
         <v>160</v>
       </c>
       <c r="N147" s="6">
-        <v>227.3</v>
+        <v>227.2</v>
       </c>
       <c r="O147" s="6">
         <v>290</v>
       </c>
       <c r="P147" s="6">
-        <v>227.62</v>
+        <v>227.3</v>
       </c>
       <c r="Q147" s="6">
-        <v>249.72</v>
+        <v>248.32</v>
       </c>
       <c r="R147" s="6">
         <f t="shared" si="0"/>
-        <v>-0.14000000000000001</v>
+        <v>-0.04</v>
       </c>
       <c r="S147" s="6">
         <f t="shared" si="1"/>
-        <v>-8.98</v>
+        <v>-8.51</v>
       </c>
       <c r="T147" s="6">
         <v>233.9</v>
@@ -12043,13 +12043,13 @@
         <v>450</v>
       </c>
       <c r="G150" s="6">
-        <v>390</v>
+        <v>380</v>
       </c>
       <c r="H150" s="6">
-        <v>404.89</v>
+        <v>394.88</v>
       </c>
       <c r="I150" s="6">
-        <v>420</v>
+        <v>410</v>
       </c>
       <c r="J150" s="6">
         <v>600</v>
@@ -12064,24 +12064,24 @@
         <v>200</v>
       </c>
       <c r="N150" s="6">
-        <v>403.28</v>
+        <v>404.02</v>
       </c>
       <c r="O150" s="6">
         <v>650</v>
       </c>
       <c r="P150" s="6">
-        <v>400.33</v>
+        <v>403.28</v>
       </c>
       <c r="Q150" s="6">
-        <v>417.21</v>
+        <v>424.39</v>
       </c>
       <c r="R150" s="6">
         <f t="shared" si="0"/>
-        <v>0.74</v>
+        <v>0.18</v>
       </c>
       <c r="S150" s="6">
         <f t="shared" si="1"/>
-        <v>-3.34</v>
+        <v>-4.8</v>
       </c>
       <c r="T150" s="6">
         <v>423.98</v>
@@ -12231,7 +12231,7 @@
         <v>323.93</v>
       </c>
       <c r="Q152" s="6">
-        <v>315.35000000000002</v>
+        <v>315.49</v>
       </c>
       <c r="R152" s="6">
         <f t="shared" si="0"/>
@@ -12239,7 +12239,7 @@
       </c>
       <c r="S152" s="6">
         <f t="shared" si="1"/>
-        <v>2.72</v>
+        <v>2.68</v>
       </c>
       <c r="T152" s="6">
         <v>315.62</v>
@@ -12380,7 +12380,7 @@
         <v>50</v>
       </c>
       <c r="N154" s="6">
-        <v>66.87</v>
+        <v>66.900000000000006</v>
       </c>
       <c r="O154" s="6">
         <v>90</v>
@@ -12393,11 +12393,11 @@
       </c>
       <c r="R154" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.04</v>
       </c>
       <c r="S154" s="6">
         <f t="shared" si="1"/>
-        <v>8.36</v>
+        <v>8.41</v>
       </c>
       <c r="T154" s="6">
         <v>62.9</v>
@@ -12465,14 +12465,14 @@
         <v>270</v>
       </c>
       <c r="P155" s="6">
-        <v>253.23</v>
+        <v>253.27</v>
       </c>
       <c r="Q155" s="6">
         <v>243.2</v>
       </c>
       <c r="R155" s="6">
         <f t="shared" ref="R155:R173" si="4">ROUND(N155/P155* 100 - 100,2)</f>
-        <v>0.02</v>
+        <v>0</v>
       </c>
       <c r="S155" s="6">
         <f t="shared" ref="S155:S173" si="5">ROUND(N155/Q155* 100 - 100,2)</f>
@@ -12623,14 +12623,14 @@
         <v>900</v>
       </c>
       <c r="P157" s="6">
-        <v>548.58000000000004</v>
+        <v>558.79</v>
       </c>
       <c r="Q157" s="6">
         <v>502.98</v>
       </c>
       <c r="R157" s="6">
         <f t="shared" si="4"/>
-        <v>1.86</v>
+        <v>0</v>
       </c>
       <c r="S157" s="6">
         <f t="shared" si="5"/>
@@ -12781,14 +12781,14 @@
         <v>490</v>
       </c>
       <c r="P159" s="6">
-        <v>318.25</v>
+        <v>320.14</v>
       </c>
       <c r="Q159" s="6">
         <v>304.39999999999998</v>
       </c>
       <c r="R159" s="6">
         <f t="shared" si="4"/>
-        <v>0.59</v>
+        <v>0</v>
       </c>
       <c r="S159" s="6">
         <f t="shared" si="5"/>
@@ -13061,40 +13061,40 @@
         <v>66</v>
       </c>
       <c r="D163" s="6">
-        <v>7.66</v>
+        <v>7.36</v>
       </c>
       <c r="E163" s="6">
-        <v>7.66</v>
+        <v>7.36</v>
       </c>
       <c r="F163" s="6">
-        <v>7.66</v>
+        <v>7.36</v>
       </c>
       <c r="G163" s="6">
-        <v>7.66</v>
+        <v>7.36</v>
       </c>
       <c r="H163" s="6">
-        <v>7.66</v>
+        <v>7.36</v>
       </c>
       <c r="I163" s="6">
-        <v>7.66</v>
+        <v>7.36</v>
       </c>
       <c r="J163" s="6">
-        <v>7.66</v>
+        <v>7.36</v>
       </c>
       <c r="K163" s="6">
-        <v>7.66</v>
+        <v>7.36</v>
       </c>
       <c r="L163" s="6">
-        <v>7.66</v>
+        <v>7.36</v>
       </c>
       <c r="M163" s="6">
-        <v>7.66</v>
+        <v>7.36</v>
       </c>
       <c r="N163" s="6">
-        <v>7.66</v>
+        <v>7.36</v>
       </c>
       <c r="O163" s="6">
-        <v>7.66</v>
+        <v>7.36</v>
       </c>
       <c r="P163" s="6">
         <v>7.66</v>
@@ -13104,11 +13104,11 @@
       </c>
       <c r="R163" s="6">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>-3.92</v>
       </c>
       <c r="S163" s="6">
         <f t="shared" si="5"/>
-        <v>58.59</v>
+        <v>52.38</v>
       </c>
       <c r="T163" s="6">
         <v>6.01</v>
@@ -13249,24 +13249,24 @@
         <v>900</v>
       </c>
       <c r="N165" s="6">
-        <v>1523.91</v>
+        <v>1526.91</v>
       </c>
       <c r="O165" s="6">
         <v>2500</v>
       </c>
       <c r="P165" s="6">
-        <v>1513.18</v>
+        <v>1523.91</v>
       </c>
       <c r="Q165" s="6">
-        <v>1385.22</v>
+        <v>1398.14</v>
       </c>
       <c r="R165" s="6">
         <f t="shared" si="4"/>
-        <v>0.71</v>
+        <v>0.2</v>
       </c>
       <c r="S165" s="6">
         <f t="shared" si="5"/>
-        <v>10.01</v>
+        <v>9.2100000000000009</v>
       </c>
       <c r="T165" s="6">
         <v>1426.49</v>
@@ -13535,54 +13535,54 @@
         <v>75</v>
       </c>
       <c r="D169" s="6">
-        <v>384.2</v>
+        <v>382.8</v>
       </c>
       <c r="E169" s="6">
-        <v>384.2</v>
+        <v>382.8</v>
       </c>
       <c r="F169" s="6">
-        <v>384.2</v>
+        <v>382.8</v>
       </c>
       <c r="G169" s="6">
-        <v>380.69</v>
+        <v>379.29</v>
       </c>
       <c r="H169" s="6">
-        <v>380.69</v>
+        <v>379.29</v>
       </c>
       <c r="I169" s="6">
-        <v>380.69</v>
+        <v>379.29</v>
       </c>
       <c r="J169" s="6">
-        <v>380.74</v>
+        <v>379.34</v>
       </c>
       <c r="K169" s="6">
-        <v>380.74</v>
+        <v>379.34</v>
       </c>
       <c r="L169" s="6">
-        <v>380.74</v>
+        <v>379.34</v>
       </c>
       <c r="M169" s="6">
-        <v>379.31</v>
+        <v>377.91</v>
       </c>
       <c r="N169" s="6">
+        <v>380.18</v>
+      </c>
+      <c r="O169" s="6">
+        <v>382.8</v>
+      </c>
+      <c r="P169" s="6">
         <v>381.67</v>
-      </c>
-      <c r="O169" s="6">
-        <v>384.2</v>
-      </c>
-      <c r="P169" s="6">
-        <v>396.06</v>
       </c>
       <c r="Q169" s="6">
         <v>264.74</v>
       </c>
       <c r="R169" s="6">
         <f t="shared" si="4"/>
-        <v>-3.63</v>
+        <v>-0.39</v>
       </c>
       <c r="S169" s="6">
         <f t="shared" si="5"/>
-        <v>44.17</v>
+        <v>43.61</v>
       </c>
       <c r="T169" s="6">
         <v>294.18</v>
@@ -13614,54 +13614,54 @@
         <v>75</v>
       </c>
       <c r="D170" s="6">
-        <v>393.5</v>
+        <v>404.9</v>
       </c>
       <c r="E170" s="6">
-        <v>393.5</v>
+        <v>404.9</v>
       </c>
       <c r="F170" s="6">
-        <v>393.5</v>
+        <v>404.9</v>
       </c>
       <c r="G170" s="6">
-        <v>391.54</v>
+        <v>401.25</v>
       </c>
       <c r="H170" s="6">
-        <v>391.54</v>
+        <v>401.25</v>
       </c>
       <c r="I170" s="6">
-        <v>391.54</v>
+        <v>401.25</v>
       </c>
       <c r="J170" s="6">
-        <v>391.55</v>
+        <v>401.55</v>
       </c>
       <c r="K170" s="6">
-        <v>391.55</v>
+        <v>401.55</v>
       </c>
       <c r="L170" s="6">
-        <v>391.55</v>
+        <v>401.55</v>
       </c>
       <c r="M170" s="6">
-        <v>390.11</v>
+        <v>399.82</v>
       </c>
       <c r="N170" s="6">
+        <v>402.08</v>
+      </c>
+      <c r="O170" s="6">
+        <v>404.9</v>
+      </c>
+      <c r="P170" s="6">
         <v>392.17</v>
-      </c>
-      <c r="O170" s="6">
-        <v>394.7</v>
-      </c>
-      <c r="P170" s="6">
-        <v>398.89</v>
       </c>
       <c r="Q170" s="6">
         <v>277.04000000000002</v>
       </c>
       <c r="R170" s="6">
         <f t="shared" si="4"/>
-        <v>-1.68</v>
+        <v>2.5299999999999998</v>
       </c>
       <c r="S170" s="6">
         <f t="shared" si="5"/>
-        <v>41.56</v>
+        <v>45.13</v>
       </c>
       <c r="T170" s="6">
         <v>306.35000000000002</v>
@@ -13693,54 +13693,54 @@
         <v>23</v>
       </c>
       <c r="D171" s="6">
-        <v>6000</v>
+        <v>5900</v>
       </c>
       <c r="E171" s="6">
-        <v>6000</v>
+        <v>5900</v>
       </c>
       <c r="F171" s="6">
-        <v>6000</v>
+        <v>5900</v>
       </c>
       <c r="G171" s="6">
-        <v>6100</v>
+        <v>6500</v>
       </c>
       <c r="H171" s="6">
-        <v>6232.62</v>
+        <v>6566.25</v>
       </c>
       <c r="I171" s="6">
-        <v>6400</v>
+        <v>6700</v>
       </c>
       <c r="J171" s="6">
+        <v>6068.4</v>
+      </c>
+      <c r="K171" s="6">
+        <v>6182.93</v>
+      </c>
+      <c r="L171" s="6">
+        <v>6418.5</v>
+      </c>
+      <c r="M171" s="6">
         <v>5835</v>
       </c>
-      <c r="K171" s="6">
-        <v>5835</v>
-      </c>
-      <c r="L171" s="6">
-        <v>5835</v>
-      </c>
-      <c r="M171" s="6">
-        <v>5600</v>
-      </c>
       <c r="N171" s="6">
-        <v>6310.76</v>
+        <v>6264.79</v>
       </c>
       <c r="O171" s="6">
         <v>7100</v>
       </c>
       <c r="P171" s="6">
-        <v>5154.16</v>
+        <v>6310.76</v>
       </c>
       <c r="Q171" s="6">
-        <v>3046.92</v>
+        <v>3028.55</v>
       </c>
       <c r="R171" s="6">
         <f t="shared" si="4"/>
-        <v>22.44</v>
+        <v>-0.73</v>
       </c>
       <c r="S171" s="6">
         <f t="shared" si="5"/>
-        <v>107.12</v>
+        <v>106.86</v>
       </c>
       <c r="T171" s="6">
         <v>3683.9</v>
@@ -14125,7 +14125,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{85D21D5C-1000-42C1-A941-AA1562148211}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{52E2B58B-4D63-474F-81B3-9B2A6675B684}">
   <dimension ref="A1:AB182"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -14321,7 +14321,7 @@
         <v>4650</v>
       </c>
       <c r="Q5" s="16">
-        <v>4669.9799999999996</v>
+        <v>4683.2700000000004</v>
       </c>
       <c r="R5" s="16">
         <v>4600</v>
@@ -14334,7 +14334,7 @@
       </c>
       <c r="U5" s="16">
         <f t="shared" ref="U5:U12" si="0">GEOMEAN(H5:T5)</f>
-        <v>4779.5057908983172</v>
+        <v>4780.550703183475</v>
       </c>
       <c r="V5" s="16">
         <f t="shared" ref="V5:V12" si="1">GEOMEAN(H39:T39)</f>
@@ -14346,11 +14346,11 @@
       </c>
       <c r="X5" s="17">
         <f t="shared" ref="X5:X12" si="3">U5/V5*100-100</f>
-        <v>0</v>
+        <v>2.1862350018437837E-2</v>
       </c>
       <c r="Y5" s="17">
         <f t="shared" ref="Y5:Y12" si="4">U5/W5*100-100</f>
-        <v>9.3692556185337423</v>
+        <v>9.3931663080096399</v>
       </c>
     </row>
     <row r="6" spans="1:25" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -14378,7 +14378,7 @@
         <v>4550</v>
       </c>
       <c r="L6" s="16">
-        <v>4533.2700000000004</v>
+        <v>4733.2700000000004</v>
       </c>
       <c r="M6" s="16">
         <v>4474.93</v>
@@ -14406,7 +14406,7 @@
       </c>
       <c r="U6" s="16">
         <f t="shared" si="0"/>
-        <v>4588.5529907886039</v>
+        <v>4608.4058658270596</v>
       </c>
       <c r="V6" s="16">
         <f t="shared" si="1"/>
@@ -14414,15 +14414,15 @@
       </c>
       <c r="W6" s="16">
         <f t="shared" si="2"/>
-        <v>4248.8815060507186</v>
+        <v>4246.8144227111061</v>
       </c>
       <c r="X6" s="17">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>0.43266090809694902</v>
       </c>
       <c r="Y6" s="17">
         <f t="shared" si="4"/>
-        <v>7.9943741489182116</v>
+        <v>8.5144159156622266</v>
       </c>
     </row>
     <row r="7" spans="1:25" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -14482,7 +14482,7 @@
       </c>
       <c r="V7" s="16">
         <f t="shared" si="1"/>
-        <v>4334.3374808766912</v>
+        <v>4327.9304043941502</v>
       </c>
       <c r="W7" s="16">
         <f t="shared" si="2"/>
@@ -14490,7 +14490,7 @@
       </c>
       <c r="X7" s="17">
         <f t="shared" si="3"/>
-        <v>-0.14782135703113397</v>
+        <v>0</v>
       </c>
       <c r="Y7" s="17">
         <f t="shared" si="4"/>
@@ -14513,13 +14513,13 @@
         <v>133</v>
       </c>
       <c r="I8" s="16">
-        <v>5100</v>
+        <v>5200</v>
       </c>
       <c r="J8" s="16">
         <v>5100</v>
       </c>
       <c r="K8" s="16">
-        <v>4800</v>
+        <v>5000</v>
       </c>
       <c r="L8" s="16">
         <v>5100</v>
@@ -14550,23 +14550,23 @@
       </c>
       <c r="U8" s="16">
         <f t="shared" si="0"/>
-        <v>4632.9616431573722</v>
+        <v>4673.003688864319</v>
       </c>
       <c r="V8" s="16">
         <f t="shared" si="1"/>
-        <v>4619.4636565713754</v>
+        <v>4632.9616431573722</v>
       </c>
       <c r="W8" s="16">
         <f t="shared" si="2"/>
-        <v>3334.3645152519698</v>
+        <v>3345.9072185542886</v>
       </c>
       <c r="X8" s="17">
         <f t="shared" si="3"/>
-        <v>0.29219813358191971</v>
+        <v>0.86428614763272549</v>
       </c>
       <c r="Y8" s="17">
         <f t="shared" si="4"/>
-        <v>38.945865755390287</v>
+        <v>39.663277659069308</v>
       </c>
     </row>
     <row r="9" spans="1:25" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -14594,7 +14594,7 @@
         <v>15800</v>
       </c>
       <c r="L9" s="16">
-        <v>15100</v>
+        <v>14800</v>
       </c>
       <c r="M9" s="16">
         <v>15099.67</v>
@@ -14622,11 +14622,11 @@
       </c>
       <c r="U9" s="16">
         <f t="shared" si="0"/>
-        <v>15375.290946417192</v>
+        <v>15336.77120139211</v>
       </c>
       <c r="V9" s="16">
         <f t="shared" si="1"/>
-        <v>15547.603515948029</v>
+        <v>15375.290946417192</v>
       </c>
       <c r="W9" s="16">
         <f t="shared" si="2"/>
@@ -14634,11 +14634,11 @@
       </c>
       <c r="X9" s="17">
         <f t="shared" si="3"/>
-        <v>-1.1082902220531139</v>
+        <v>-0.25053018612345568</v>
       </c>
       <c r="Y9" s="17">
         <f t="shared" si="4"/>
-        <v>23.818889718518491</v>
+        <v>23.508686023650682</v>
       </c>
     </row>
     <row r="10" spans="1:25" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -14698,19 +14698,19 @@
       </c>
       <c r="V10" s="16">
         <f t="shared" si="1"/>
-        <v>10626.960981644181</v>
+        <v>10666.943602772601</v>
       </c>
       <c r="W10" s="16">
         <f t="shared" si="2"/>
-        <v>9176.2396627494836</v>
+        <v>9224.9312568359583</v>
       </c>
       <c r="X10" s="17">
         <f t="shared" si="3"/>
-        <v>0.37623758285630515</v>
+        <v>0</v>
       </c>
       <c r="Y10" s="17">
         <f t="shared" si="4"/>
-        <v>16.245259439708846</v>
+        <v>15.63168663038077</v>
       </c>
     </row>
     <row r="11" spans="1:25" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -14753,7 +14753,7 @@
         <v>17100</v>
       </c>
       <c r="Q11" s="16">
-        <v>16967.86</v>
+        <v>17034.93</v>
       </c>
       <c r="R11" s="16">
         <v>17100</v>
@@ -14766,23 +14766,23 @@
       </c>
       <c r="U11" s="16">
         <f t="shared" si="0"/>
-        <v>17148.059394865042</v>
+        <v>17153.263928695029</v>
       </c>
       <c r="V11" s="16">
         <f t="shared" si="1"/>
-        <v>17117.512199952787</v>
+        <v>17148.059394865042</v>
       </c>
       <c r="W11" s="16">
         <f t="shared" si="2"/>
-        <v>14593.756964569429</v>
+        <v>14586.249860123879</v>
       </c>
       <c r="X11" s="17">
         <f t="shared" si="3"/>
-        <v>0.17845580920537429</v>
+        <v>3.0350570348190331E-2</v>
       </c>
       <c r="Y11" s="17">
         <f t="shared" si="4"/>
-        <v>17.502706372984832</v>
+        <v>17.598862580771325</v>
       </c>
     </row>
     <row r="12" spans="1:25" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -14831,14 +14831,14 @@
         <v>11500</v>
       </c>
       <c r="S12" s="16">
-        <v>11000</v>
+        <v>10700</v>
       </c>
       <c r="T12" s="16">
         <v>12240.64</v>
       </c>
       <c r="U12" s="16">
         <f t="shared" si="0"/>
-        <v>11117.297564429658</v>
+        <v>11083.193281913298</v>
       </c>
       <c r="V12" s="16">
         <f t="shared" si="1"/>
@@ -14846,15 +14846,15 @@
       </c>
       <c r="W12" s="16">
         <f t="shared" si="2"/>
-        <v>9406.1881883517817</v>
+        <v>9400.5859188821632</v>
       </c>
       <c r="X12" s="17">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>-0.30676774025981501</v>
       </c>
       <c r="Y12" s="17">
         <f t="shared" si="4"/>
-        <v>18.191315566031747</v>
+        <v>17.898962655630044</v>
       </c>
     </row>
     <row r="13" spans="1:25" x14ac:dyDescent="0.25">
@@ -15018,25 +15018,25 @@
       </c>
       <c r="C17" s="35"/>
       <c r="D17" s="16">
-        <v>1579.04</v>
+        <v>1544.89</v>
       </c>
       <c r="E17" s="16">
-        <v>1519.98</v>
+        <v>1517.97</v>
       </c>
       <c r="F17" s="16">
         <v>1650</v>
       </c>
       <c r="G17" s="16">
-        <v>1646.66</v>
+        <v>1630</v>
       </c>
       <c r="H17" s="16">
-        <v>1649.98</v>
+        <v>1659.51</v>
       </c>
       <c r="I17" s="16">
         <v>1600</v>
       </c>
       <c r="J17" s="16">
-        <v>1628.33</v>
+        <v>1618.33</v>
       </c>
       <c r="K17" s="16">
         <v>1656.65</v>
@@ -15045,10 +15045,10 @@
         <v>1659.94</v>
       </c>
       <c r="M17" s="16">
-        <v>1479.57</v>
+        <v>1481.1</v>
       </c>
       <c r="N17" s="16">
-        <v>1563.33</v>
+        <v>1564.99</v>
       </c>
       <c r="O17" s="16">
         <v>1650</v>
@@ -15057,7 +15057,7 @@
         <v>1523.33</v>
       </c>
       <c r="Q17" s="16">
-        <v>1633.16</v>
+        <v>1610.95</v>
       </c>
       <c r="R17" s="16">
         <v>1500</v>
@@ -15070,21 +15070,21 @@
       </c>
       <c r="U17" s="16">
         <f>GEOMEAN(D17:T17)</f>
-        <v>1595.9159403409981</v>
+        <v>1591.6637602185144</v>
       </c>
       <c r="V17" s="16">
-        <v>1600.39</v>
+        <v>1595.92</v>
       </c>
       <c r="W17" s="16">
-        <v>1393.35</v>
+        <v>1390.32</v>
       </c>
       <c r="X17" s="17">
         <f>U17/V17*100-100</f>
-        <v>-0.27956058579484022</v>
+        <v>-0.26669505874265553</v>
       </c>
       <c r="Y17" s="17">
         <f>U17/W17*100-100</f>
-        <v>14.538051483187871</v>
+        <v>14.481828659482304</v>
       </c>
     </row>
     <row r="18" spans="1:28" x14ac:dyDescent="0.25">
@@ -15620,14 +15620,14 @@
         <v>2121.7316339927452</v>
       </c>
       <c r="V28" s="16">
-        <v>2115.52</v>
+        <v>2121.73</v>
       </c>
       <c r="W28" s="16">
         <v>1975.63</v>
       </c>
       <c r="X28" s="17">
         <f>U28/V28*100-100</f>
-        <v>0.29362208784343125</v>
+        <v>7.7012284549482501E-5</v>
       </c>
       <c r="Y28" s="17">
         <f>U28/W28*100-100</f>
@@ -15700,14 +15700,14 @@
         <v>1320.8632031159254</v>
       </c>
       <c r="V29" s="16">
-        <v>1317.05</v>
+        <v>1320.86</v>
       </c>
       <c r="W29" s="16">
         <v>1209.7</v>
       </c>
       <c r="X29" s="17">
         <f>U29/V29*100-100</f>
-        <v>0.28952607083448356</v>
+        <v>2.4250230346467561E-4</v>
       </c>
       <c r="Y29" s="17">
         <f>U29/W29*100-100</f>
@@ -15780,14 +15780,14 @@
         <v>1918.2806250596295</v>
       </c>
       <c r="V30" s="16">
-        <v>1915.7</v>
+        <v>1918.28</v>
       </c>
       <c r="W30" s="16">
         <v>1754.23</v>
       </c>
       <c r="X30" s="17">
         <f>U30/V30*100-100</f>
-        <v>0.13470924777519144</v>
+        <v>3.2584379212607928E-5</v>
       </c>
       <c r="Y30" s="17">
         <f>U30/W30*100-100</f>
@@ -15860,14 +15860,14 @@
         <v>288.79072542131092</v>
       </c>
       <c r="V31" s="16">
-        <v>287.92</v>
+        <v>288.79000000000002</v>
       </c>
       <c r="W31" s="16">
         <v>278.64999999999998</v>
       </c>
       <c r="X31" s="17">
         <f>U31/V31*100-100</f>
-        <v>0.30241922107214236</v>
+        <v>2.5119336225998268E-4</v>
       </c>
       <c r="Y31" s="17">
         <f>U31/W31*100-100</f>
@@ -15998,7 +15998,7 @@
         <v>1453.31</v>
       </c>
       <c r="G34" s="26">
-        <v>1325</v>
+        <v>1350</v>
       </c>
       <c r="H34" s="26">
         <v>1300</v>
@@ -16007,22 +16007,22 @@
         <v>1350</v>
       </c>
       <c r="J34" s="26">
-        <v>1275</v>
+        <v>1300</v>
       </c>
       <c r="K34" s="26">
         <v>1223.33</v>
       </c>
       <c r="L34" s="26">
-        <v>1312.44</v>
+        <v>1337.44</v>
       </c>
       <c r="M34" s="26">
-        <v>1283.1099999999999</v>
+        <v>1266.6099999999999</v>
       </c>
       <c r="N34" s="26">
-        <v>1464.99</v>
+        <v>1440</v>
       </c>
       <c r="O34" s="26">
-        <v>1459.93</v>
+        <v>1453.33</v>
       </c>
       <c r="P34" s="26">
         <v>1488.57</v>
@@ -16031,10 +16031,10 @@
         <v>1408.28</v>
       </c>
       <c r="R34" s="26">
-        <v>1459.93</v>
+        <v>1469.93</v>
       </c>
       <c r="S34" s="26">
-        <v>1393.3</v>
+        <v>1460</v>
       </c>
       <c r="T34" s="26">
         <v>1384.97</v>
@@ -16043,13 +16043,13 @@
         <v>1450</v>
       </c>
       <c r="V34" s="25">
+        <v>1385.3242635355812</v>
+      </c>
+      <c r="W34" s="25">
         <v>1379.153945812214</v>
       </c>
-      <c r="W34" s="25">
-        <v>1379.5286919751202</v>
-      </c>
       <c r="X34" s="41">
-        <v>-0.03</v>
+        <v>0.45</v>
       </c>
       <c r="Y34" s="42"/>
       <c r="Z34" s="20"/>
@@ -16086,7 +16086,7 @@
         <v>164.92</v>
       </c>
       <c r="K35" s="26">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="L35" s="26">
         <v>159.16</v>
@@ -16095,7 +16095,7 @@
         <v>148.31</v>
       </c>
       <c r="N35" s="26">
-        <v>186.46</v>
+        <v>185.08</v>
       </c>
       <c r="O35" s="26">
         <v>187.48</v>
@@ -16107,25 +16107,25 @@
         <v>170</v>
       </c>
       <c r="R35" s="26">
-        <v>170.24</v>
+        <v>171.93</v>
       </c>
       <c r="S35" s="26">
         <v>165</v>
       </c>
       <c r="T35" s="26">
-        <v>182.5</v>
+        <v>187.49</v>
       </c>
       <c r="U35" s="26">
         <v>180</v>
       </c>
       <c r="V35" s="25">
+        <v>170.07717571702926</v>
+      </c>
+      <c r="W35" s="25">
         <v>169.98493620622341</v>
       </c>
-      <c r="W35" s="25">
-        <v>170.02607066007207</v>
-      </c>
       <c r="X35" s="41">
-        <v>-0.02</v>
+        <v>0.05</v>
       </c>
       <c r="Y35" s="42"/>
       <c r="Z35" s="20"/>
@@ -16392,7 +16392,7 @@
         <v>4349.71</v>
       </c>
       <c r="P41" s="1">
-        <v>4250</v>
+        <v>4200</v>
       </c>
       <c r="Q41" s="1" t="s">
         <v>133</v>
@@ -16448,7 +16448,7 @@
         <v>133</v>
       </c>
       <c r="Q42" s="1">
-        <v>4700</v>
+        <v>4796.9799999999996</v>
       </c>
       <c r="R42" s="1">
         <v>5000</v>
@@ -16492,7 +16492,7 @@
         <v>15099.67</v>
       </c>
       <c r="N43" s="1">
-        <v>14831.45</v>
+        <v>13566.34</v>
       </c>
       <c r="O43" s="1" t="s">
         <v>133</v>
@@ -16530,7 +16530,7 @@
         <v>133</v>
       </c>
       <c r="I44" s="1">
-        <v>10600</v>
+        <v>11000</v>
       </c>
       <c r="J44" s="1">
         <v>11000</v>
@@ -16539,7 +16539,7 @@
         <v>10700</v>
       </c>
       <c r="L44" s="1">
-        <v>10800</v>
+        <v>10700</v>
       </c>
       <c r="M44" s="1">
         <v>10149.879999999999</v>
@@ -16551,13 +16551,13 @@
         <v>10749.88</v>
       </c>
       <c r="P44" s="1">
-        <v>10500</v>
+        <v>10400</v>
       </c>
       <c r="Q44" s="1">
-        <v>10491.59</v>
+        <v>10764.11</v>
       </c>
       <c r="R44" s="1">
-        <v>10700</v>
+        <v>10633.23</v>
       </c>
       <c r="S44" s="1" t="s">
         <v>133</v>
@@ -16583,7 +16583,7 @@
         <v>17000</v>
       </c>
       <c r="I45" s="1">
-        <v>17200</v>
+        <v>17500</v>
       </c>
       <c r="J45" s="1">
         <v>17250</v>
@@ -16592,13 +16592,13 @@
         <v>17200</v>
       </c>
       <c r="L45" s="1">
-        <v>17300</v>
+        <v>17200</v>
       </c>
       <c r="M45" s="1">
         <v>16099.69</v>
       </c>
       <c r="N45" s="1">
-        <v>16999.8</v>
+        <v>17166.599999999999</v>
       </c>
       <c r="O45" s="1">
         <v>17149.93</v>
@@ -16607,10 +16607,10 @@
         <v>17100</v>
       </c>
       <c r="Q45" s="1">
-        <v>17034.93</v>
+        <v>16967.86</v>
       </c>
       <c r="R45" s="1">
-        <v>17000</v>
+        <v>17100</v>
       </c>
       <c r="S45" s="1">
         <v>17500</v>
@@ -16763,7 +16763,7 @@
         <v>133</v>
       </c>
       <c r="P48" s="1">
-        <v>4120</v>
+        <v>4100</v>
       </c>
       <c r="Q48" s="1" t="s">
         <v>133</v>
@@ -16875,7 +16875,7 @@
         <v>3613.28</v>
       </c>
       <c r="R50" s="1">
-        <v>3400</v>
+        <v>3483.25</v>
       </c>
       <c r="S50" s="1" t="s">
         <v>133</v>
@@ -16960,7 +16960,7 @@
         <v>9100</v>
       </c>
       <c r="K52" s="1">
-        <v>9200</v>
+        <v>9700</v>
       </c>
       <c r="L52" s="1">
         <v>9300</v>
@@ -17007,7 +17007,7 @@
         <v>13500</v>
       </c>
       <c r="I53" s="1">
-        <v>15000</v>
+        <v>14900</v>
       </c>
       <c r="J53" s="1">
         <v>14900</v>
@@ -17090,7 +17090,7 @@
         <v>9000</v>
       </c>
       <c r="S54" s="1">
-        <v>9350</v>
+        <v>9300</v>
       </c>
       <c r="T54" s="1">
         <v>9699.66</v>

</xml_diff>